<commit_message>
Step 5: Excel databook with live formulas, checks and native charts
- databook/build_databook.py builds 13 tabs from outputs/tables/:
  cover, contents, basis of preparation, reconciliation, 4a-4g, Q&A
  log and checks; inputs in blue, every total/share/growth/check a
  formula; £ stored in pounds and shown in £'000
- databook/recalc.py recalculates with LibreOffice headless and scans
  every cell: 901 formulas, 0 errors, 53/53 checks TRUE
- cell_map.json lets the tests compare 147 key figures with
  outputs/tables/ to the penny
- saved tables rounded to 6 dp and tie-breaks added so runs are
  byte-identical
- 5 new tests (84 in total); decisions D18-D20

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LpN25NXzSEvizAa4wBvUc3
</commit_message>
<xml_diff>
--- a/databook/Northbridge_Databook.xlsx
+++ b/databook/Northbridge_Databook.xlsx
@@ -2900,11 +2900,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="77968525"/>
-        <c:axId val="61733620"/>
+        <c:axId val="68182179"/>
+        <c:axId val="30665427"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="77968525"/>
+        <c:axId val="68182179"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2970,7 +2970,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61733620"/>
+        <c:crossAx val="30665427"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2978,7 +2978,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61733620"/>
+        <c:axId val="30665427"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3044,7 +3044,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77968525"/>
+        <c:crossAx val="68182179"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3419,11 +3419,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="25029982"/>
-        <c:axId val="53280423"/>
+        <c:axId val="92032456"/>
+        <c:axId val="51481830"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25029982"/>
+        <c:axId val="92032456"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3489,7 +3489,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53280423"/>
+        <c:crossAx val="51481830"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3497,7 +3497,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="53280423"/>
+        <c:axId val="51481830"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3563,7 +3563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25029982"/>
+        <c:crossAx val="92032456"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4051,11 +4051,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="13652970"/>
-        <c:axId val="11613285"/>
+        <c:axId val="80391956"/>
+        <c:axId val="61916199"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="13652970"/>
+        <c:axId val="80391956"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4121,7 +4121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11613285"/>
+        <c:crossAx val="61916199"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4129,7 +4129,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11613285"/>
+        <c:axId val="61916199"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4195,7 +4195,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13652970"/>
+        <c:crossAx val="80391956"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4656,11 +4656,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="97048973"/>
-        <c:axId val="15051131"/>
+        <c:axId val="11610500"/>
+        <c:axId val="97597414"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="97048973"/>
+        <c:axId val="11610500"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4726,7 +4726,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15051131"/>
+        <c:crossAx val="97597414"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4734,7 +4734,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="15051131"/>
+        <c:axId val="97597414"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4800,7 +4800,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97048973"/>
+        <c:crossAx val="11610500"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5157,11 +5157,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="69470306"/>
-        <c:axId val="19174714"/>
+        <c:axId val="99355520"/>
+        <c:axId val="79132325"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="69470306"/>
+        <c:axId val="99355520"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5227,7 +5227,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19174714"/>
+        <c:crossAx val="79132325"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5235,7 +5235,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19174714"/>
+        <c:axId val="79132325"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.1"/>
@@ -5303,7 +5303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69470306"/>
+        <c:crossAx val="99355520"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5890,11 +5890,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="2956759"/>
-        <c:axId val="2533916"/>
+        <c:axId val="90034550"/>
+        <c:axId val="44332542"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2956759"/>
+        <c:axId val="90034550"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5926,7 +5926,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2533916"/>
+        <c:crossAx val="44332542"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5934,7 +5934,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2533916"/>
+        <c:axId val="44332542"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="25000000"/>
@@ -6001,7 +6001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2956759"/>
+        <c:crossAx val="90034550"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6489,11 +6489,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="56365667"/>
-        <c:axId val="80053178"/>
+        <c:axId val="47346770"/>
+        <c:axId val="39380636"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="56365667"/>
+        <c:axId val="47346770"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6559,7 +6559,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80053178"/>
+        <c:crossAx val="39380636"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6567,7 +6567,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80053178"/>
+        <c:axId val="39380636"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6633,7 +6633,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56365667"/>
+        <c:crossAx val="47346770"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6819,11 +6819,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="95184699"/>
-        <c:axId val="82241058"/>
+        <c:axId val="62505300"/>
+        <c:axId val="49705050"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="95184699"/>
+        <c:axId val="62505300"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6855,7 +6855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82241058"/>
+        <c:crossAx val="49705050"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6863,7 +6863,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="82241058"/>
+        <c:axId val="49705050"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6929,7 +6929,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95184699"/>
+        <c:crossAx val="62505300"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -17935,31 +17935,31 @@
         <v>1</v>
       </c>
       <c r="M43" s="27" t="n">
-        <v>0.966666666666667</v>
+        <v>0.96666667</v>
       </c>
       <c r="N43" s="27" t="n">
         <v>0.95</v>
       </c>
       <c r="O43" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="P43" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="Q43" s="27" t="n">
         <v>0.9</v>
       </c>
       <c r="R43" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="S43" s="27" t="n">
         <v>0.85</v>
       </c>
       <c r="T43" s="27" t="n">
-        <v>0.833333333333334</v>
+        <v>0.83333333</v>
       </c>
       <c r="U43" s="27" t="n">
-        <v>0.816666666666667</v>
+        <v>0.81666667</v>
       </c>
       <c r="V43" s="27" t="n">
         <v>0.8</v>
@@ -17974,31 +17974,31 @@
         <v>0.8</v>
       </c>
       <c r="Z43" s="27" t="n">
-        <v>0.783333333333333</v>
+        <v>0.78333333</v>
       </c>
       <c r="AA43" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="AB43" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="AC43" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="AD43" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="AE43" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="AF43" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="AG43" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="AH43" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="AI43" s="27" t="n">
         <v>0.75</v>
@@ -18010,7 +18010,7 @@
         <v>0.75</v>
       </c>
       <c r="AL43" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18161,88 +18161,88 @@
         <v>1</v>
       </c>
       <c r="K45" s="27" t="n">
-        <v>0.972222222222222</v>
+        <v>0.97222222</v>
       </c>
       <c r="L45" s="27" t="n">
-        <v>0.972222222222222</v>
+        <v>0.97222222</v>
       </c>
       <c r="M45" s="27" t="n">
-        <v>0.944444444444444</v>
+        <v>0.94444444</v>
       </c>
       <c r="N45" s="27" t="n">
-        <v>0.944444444444444</v>
+        <v>0.94444444</v>
       </c>
       <c r="O45" s="27" t="n">
-        <v>0.944444444444444</v>
+        <v>0.94444444</v>
       </c>
       <c r="P45" s="27" t="n">
-        <v>0.944444444444444</v>
+        <v>0.94444444</v>
       </c>
       <c r="Q45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="R45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="S45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="T45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="U45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="V45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="W45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="X45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="Y45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="Z45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="AA45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="AB45" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="AC45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AD45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AE45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AF45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AG45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AH45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AI45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AJ45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AK45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="AL45" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18262,103 +18262,103 @@
         <v>1</v>
       </c>
       <c r="F46" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="G46" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="H46" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="I46" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="J46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="K46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="L46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="M46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="N46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="O46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="P46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="Q46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="R46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="S46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="T46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="U46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="V46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="W46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="X46" s="27" t="n">
-        <v>0.930232558139535</v>
+        <v>0.93023256</v>
       </c>
       <c r="Y46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="Z46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AA46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AB46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AC46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AD46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AE46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AF46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AG46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AH46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AI46" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AJ46" s="27" t="n">
-        <v>0.86046511627907</v>
+        <v>0.86046512</v>
       </c>
       <c r="AK46" s="27" t="n">
-        <v>0.86046511627907</v>
+        <v>0.86046512</v>
       </c>
       <c r="AL46" s="27" t="n">
-        <v>0.86046511627907</v>
+        <v>0.86046512</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18497,100 +18497,100 @@
         <v>1</v>
       </c>
       <c r="G48" s="27" t="n">
-        <v>0.973684210526316</v>
+        <v>0.97368421</v>
       </c>
       <c r="H48" s="27" t="n">
-        <v>0.973684210526316</v>
+        <v>0.97368421</v>
       </c>
       <c r="I48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="J48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="K48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="L48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="M48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="N48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="O48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="P48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="Q48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="R48" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="S48" s="27" t="n">
-        <v>0.921052631578947</v>
+        <v>0.92105263</v>
       </c>
       <c r="T48" s="27" t="n">
-        <v>0.921052631578947</v>
+        <v>0.92105263</v>
       </c>
       <c r="U48" s="27" t="n">
-        <v>0.921052631578947</v>
+        <v>0.92105263</v>
       </c>
       <c r="V48" s="27" t="n">
-        <v>0.894736842105263</v>
+        <v>0.89473684</v>
       </c>
       <c r="W48" s="27" t="n">
-        <v>0.894736842105263</v>
+        <v>0.89473684</v>
       </c>
       <c r="X48" s="27" t="n">
-        <v>0.894736842105263</v>
+        <v>0.89473684</v>
       </c>
       <c r="Y48" s="27" t="n">
-        <v>0.894736842105263</v>
+        <v>0.89473684</v>
       </c>
       <c r="Z48" s="27" t="n">
-        <v>0.894736842105263</v>
+        <v>0.89473684</v>
       </c>
       <c r="AA48" s="27" t="n">
-        <v>0.894736842105263</v>
+        <v>0.89473684</v>
       </c>
       <c r="AB48" s="27" t="n">
-        <v>0.868421052631579</v>
+        <v>0.86842105</v>
       </c>
       <c r="AC48" s="27" t="n">
-        <v>0.868421052631579</v>
+        <v>0.86842105</v>
       </c>
       <c r="AD48" s="27" t="n">
-        <v>0.868421052631579</v>
+        <v>0.86842105</v>
       </c>
       <c r="AE48" s="27" t="n">
-        <v>0.842105263157895</v>
+        <v>0.84210526</v>
       </c>
       <c r="AF48" s="27" t="n">
-        <v>0.815789473684211</v>
+        <v>0.81578947</v>
       </c>
       <c r="AG48" s="27" t="n">
-        <v>0.815789473684211</v>
+        <v>0.81578947</v>
       </c>
       <c r="AH48" s="27" t="n">
-        <v>0.815789473684211</v>
+        <v>0.81578947</v>
       </c>
       <c r="AI48" s="27" t="n">
-        <v>0.815789473684211</v>
+        <v>0.81578947</v>
       </c>
       <c r="AJ48" s="27" t="n">
-        <v>0.815789473684211</v>
+        <v>0.81578947</v>
       </c>
       <c r="AK48" s="27" t="n">
-        <v>0.815789473684211</v>
+        <v>0.81578947</v>
       </c>
       <c r="AL48" s="27" t="n">
-        <v>0.815789473684211</v>
+        <v>0.81578947</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18601,112 +18601,112 @@
         <v>1</v>
       </c>
       <c r="C49" s="27" t="n">
-        <v>0.975609756097561</v>
+        <v>0.97560976</v>
       </c>
       <c r="D49" s="27" t="n">
-        <v>0.975609756097561</v>
+        <v>0.97560976</v>
       </c>
       <c r="E49" s="27" t="n">
-        <v>0.975609756097561</v>
+        <v>0.97560976</v>
       </c>
       <c r="F49" s="27" t="n">
-        <v>0.951219512195122</v>
+        <v>0.95121951</v>
       </c>
       <c r="G49" s="27" t="n">
-        <v>0.951219512195122</v>
+        <v>0.95121951</v>
       </c>
       <c r="H49" s="27" t="n">
-        <v>0.951219512195122</v>
+        <v>0.95121951</v>
       </c>
       <c r="I49" s="27" t="n">
-        <v>0.951219512195122</v>
+        <v>0.95121951</v>
       </c>
       <c r="J49" s="27" t="n">
-        <v>0.926829268292683</v>
+        <v>0.92682927</v>
       </c>
       <c r="K49" s="27" t="n">
-        <v>0.926829268292683</v>
+        <v>0.92682927</v>
       </c>
       <c r="L49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="M49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="N49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="O49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="P49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="Q49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="R49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="S49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="T49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="U49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="V49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="W49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="X49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="Y49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="Z49" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="AA49" s="27" t="n">
-        <v>0.878048780487805</v>
+        <v>0.87804878</v>
       </c>
       <c r="AB49" s="27" t="n">
-        <v>0.878048780487805</v>
+        <v>0.87804878</v>
       </c>
       <c r="AC49" s="27" t="n">
-        <v>0.878048780487805</v>
+        <v>0.87804878</v>
       </c>
       <c r="AD49" s="27" t="n">
-        <v>0.878048780487805</v>
+        <v>0.87804878</v>
       </c>
       <c r="AE49" s="27" t="n">
-        <v>0.853658536585366</v>
+        <v>0.85365854</v>
       </c>
       <c r="AF49" s="27" t="n">
-        <v>0.829268292682927</v>
+        <v>0.82926829</v>
       </c>
       <c r="AG49" s="27" t="n">
-        <v>0.829268292682927</v>
+        <v>0.82926829</v>
       </c>
       <c r="AH49" s="27" t="n">
-        <v>0.829268292682927</v>
+        <v>0.82926829</v>
       </c>
       <c r="AI49" s="27" t="n">
-        <v>0.829268292682927</v>
+        <v>0.82926829</v>
       </c>
       <c r="AJ49" s="27" t="n">
-        <v>0.829268292682927</v>
+        <v>0.82926829</v>
       </c>
       <c r="AK49" s="27" t="n">
-        <v>0.829268292682927</v>
+        <v>0.82926829</v>
       </c>
       <c r="AL49" s="27" t="n">
-        <v>0.829268292682927</v>
+        <v>0.82926829</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18750,79 +18750,79 @@
         <v>1</v>
       </c>
       <c r="N50" s="27" t="n">
-        <v>0.983050847457627</v>
+        <v>0.98305085</v>
       </c>
       <c r="O50" s="27" t="n">
-        <v>0.966101694915254</v>
+        <v>0.96610169</v>
       </c>
       <c r="P50" s="27" t="n">
-        <v>0.966101694915254</v>
+        <v>0.96610169</v>
       </c>
       <c r="Q50" s="27" t="n">
-        <v>0.966101694915254</v>
+        <v>0.96610169</v>
       </c>
       <c r="R50" s="27" t="n">
-        <v>0.966101694915254</v>
+        <v>0.96610169</v>
       </c>
       <c r="S50" s="27" t="n">
-        <v>0.966101694915254</v>
+        <v>0.96610169</v>
       </c>
       <c r="T50" s="27" t="n">
-        <v>0.966101694915254</v>
+        <v>0.96610169</v>
       </c>
       <c r="U50" s="27" t="n">
-        <v>0.949152542372881</v>
+        <v>0.94915254</v>
       </c>
       <c r="V50" s="27" t="n">
-        <v>0.949152542372881</v>
+        <v>0.94915254</v>
       </c>
       <c r="W50" s="27" t="n">
-        <v>0.932203389830508</v>
+        <v>0.93220339</v>
       </c>
       <c r="X50" s="27" t="n">
-        <v>0.932203389830508</v>
+        <v>0.93220339</v>
       </c>
       <c r="Y50" s="27" t="n">
-        <v>0.932203389830508</v>
+        <v>0.93220339</v>
       </c>
       <c r="Z50" s="27" t="n">
-        <v>0.932203389830508</v>
+        <v>0.93220339</v>
       </c>
       <c r="AA50" s="27" t="n">
-        <v>0.932203389830508</v>
+        <v>0.93220339</v>
       </c>
       <c r="AB50" s="27" t="n">
-        <v>0.915254237288136</v>
+        <v>0.91525424</v>
       </c>
       <c r="AC50" s="27" t="n">
-        <v>0.898305084745763</v>
+        <v>0.89830508</v>
       </c>
       <c r="AD50" s="27" t="n">
-        <v>0.898305084745763</v>
+        <v>0.89830508</v>
       </c>
       <c r="AE50" s="27" t="n">
-        <v>0.898305084745763</v>
+        <v>0.89830508</v>
       </c>
       <c r="AF50" s="27" t="n">
-        <v>0.898305084745763</v>
+        <v>0.89830508</v>
       </c>
       <c r="AG50" s="27" t="n">
-        <v>0.898305084745763</v>
+        <v>0.89830508</v>
       </c>
       <c r="AH50" s="27" t="n">
-        <v>0.864406779661017</v>
+        <v>0.86440678</v>
       </c>
       <c r="AI50" s="27" t="n">
-        <v>0.864406779661017</v>
+        <v>0.86440678</v>
       </c>
       <c r="AJ50" s="27" t="n">
-        <v>0.864406779661017</v>
+        <v>0.86440678</v>
       </c>
       <c r="AK50" s="27" t="n">
-        <v>0.847457627118644</v>
+        <v>0.84745763</v>
       </c>
       <c r="AL50" s="27" t="n">
-        <v>0.847457627118644</v>
+        <v>0.84745763</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18845,100 +18845,100 @@
         <v>1</v>
       </c>
       <c r="G51" s="27" t="n">
-        <v>0.948275862068966</v>
+        <v>0.94827586</v>
       </c>
       <c r="H51" s="27" t="n">
-        <v>0.948275862068966</v>
+        <v>0.94827586</v>
       </c>
       <c r="I51" s="27" t="n">
-        <v>0.931034482758621</v>
+        <v>0.93103448</v>
       </c>
       <c r="J51" s="27" t="n">
-        <v>0.931034482758621</v>
+        <v>0.93103448</v>
       </c>
       <c r="K51" s="27" t="n">
-        <v>0.913793103448276</v>
+        <v>0.9137931</v>
       </c>
       <c r="L51" s="27" t="n">
-        <v>0.896551724137931</v>
+        <v>0.89655172</v>
       </c>
       <c r="M51" s="27" t="n">
-        <v>0.879310344827586</v>
+        <v>0.87931034</v>
       </c>
       <c r="N51" s="27" t="n">
-        <v>0.879310344827586</v>
+        <v>0.87931034</v>
       </c>
       <c r="O51" s="27" t="n">
-        <v>0.879310344827586</v>
+        <v>0.87931034</v>
       </c>
       <c r="P51" s="27" t="n">
-        <v>0.879310344827586</v>
+        <v>0.87931034</v>
       </c>
       <c r="Q51" s="27" t="n">
-        <v>0.862068965517241</v>
+        <v>0.86206897</v>
       </c>
       <c r="R51" s="27" t="n">
-        <v>0.862068965517241</v>
+        <v>0.86206897</v>
       </c>
       <c r="S51" s="27" t="n">
-        <v>0.827586206896552</v>
+        <v>0.82758621</v>
       </c>
       <c r="T51" s="27" t="n">
-        <v>0.827586206896552</v>
+        <v>0.82758621</v>
       </c>
       <c r="U51" s="27" t="n">
-        <v>0.793103448275862</v>
+        <v>0.79310345</v>
       </c>
       <c r="V51" s="27" t="n">
-        <v>0.793103448275862</v>
+        <v>0.79310345</v>
       </c>
       <c r="W51" s="27" t="n">
-        <v>0.775862068965517</v>
+        <v>0.77586207</v>
       </c>
       <c r="X51" s="27" t="n">
-        <v>0.758620689655172</v>
+        <v>0.75862069</v>
       </c>
       <c r="Y51" s="27" t="n">
-        <v>0.758620689655172</v>
+        <v>0.75862069</v>
       </c>
       <c r="Z51" s="27" t="n">
-        <v>0.741379310344828</v>
+        <v>0.74137931</v>
       </c>
       <c r="AA51" s="27" t="n">
-        <v>0.741379310344828</v>
+        <v>0.74137931</v>
       </c>
       <c r="AB51" s="27" t="n">
-        <v>0.724137931034483</v>
+        <v>0.72413793</v>
       </c>
       <c r="AC51" s="27" t="n">
-        <v>0.706896551724138</v>
+        <v>0.70689655</v>
       </c>
       <c r="AD51" s="27" t="n">
-        <v>0.689655172413793</v>
+        <v>0.68965517</v>
       </c>
       <c r="AE51" s="27" t="n">
-        <v>0.689655172413793</v>
+        <v>0.68965517</v>
       </c>
       <c r="AF51" s="27" t="n">
-        <v>0.689655172413793</v>
+        <v>0.68965517</v>
       </c>
       <c r="AG51" s="27" t="n">
-        <v>0.672413793103448</v>
+        <v>0.67241379</v>
       </c>
       <c r="AH51" s="27" t="n">
-        <v>0.672413793103448</v>
+        <v>0.67241379</v>
       </c>
       <c r="AI51" s="27" t="n">
-        <v>0.672413793103448</v>
+        <v>0.67241379</v>
       </c>
       <c r="AJ51" s="27" t="n">
-        <v>0.672413793103448</v>
+        <v>0.67241379</v>
       </c>
       <c r="AK51" s="27" t="n">
-        <v>0.672413793103448</v>
+        <v>0.67241379</v>
       </c>
       <c r="AL51" s="27" t="n">
-        <v>0.672413793103448</v>
+        <v>0.67241379</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18970,91 +18970,91 @@
         <v>1</v>
       </c>
       <c r="J52" s="27" t="n">
-        <v>0.980769230769231</v>
+        <v>0.98076923</v>
       </c>
       <c r="K52" s="27" t="n">
-        <v>0.961538461538462</v>
+        <v>0.96153846</v>
       </c>
       <c r="L52" s="27" t="n">
-        <v>0.961538461538462</v>
+        <v>0.96153846</v>
       </c>
       <c r="M52" s="27" t="n">
-        <v>0.923076923076923</v>
+        <v>0.92307692</v>
       </c>
       <c r="N52" s="27" t="n">
-        <v>0.923076923076923</v>
+        <v>0.92307692</v>
       </c>
       <c r="O52" s="27" t="n">
-        <v>0.923076923076923</v>
+        <v>0.92307692</v>
       </c>
       <c r="P52" s="27" t="n">
-        <v>0.903846153846154</v>
+        <v>0.90384615</v>
       </c>
       <c r="Q52" s="27" t="n">
-        <v>0.903846153846154</v>
+        <v>0.90384615</v>
       </c>
       <c r="R52" s="27" t="n">
-        <v>0.865384615384615</v>
+        <v>0.86538462</v>
       </c>
       <c r="S52" s="27" t="n">
-        <v>0.865384615384615</v>
+        <v>0.86538462</v>
       </c>
       <c r="T52" s="27" t="n">
-        <v>0.865384615384615</v>
+        <v>0.86538462</v>
       </c>
       <c r="U52" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="V52" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="W52" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="X52" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="Y52" s="27" t="n">
-        <v>0.826923076923077</v>
+        <v>0.82692308</v>
       </c>
       <c r="Z52" s="27" t="n">
-        <v>0.826923076923077</v>
+        <v>0.82692308</v>
       </c>
       <c r="AA52" s="27" t="n">
-        <v>0.826923076923077</v>
+        <v>0.82692308</v>
       </c>
       <c r="AB52" s="27" t="n">
-        <v>0.826923076923077</v>
+        <v>0.82692308</v>
       </c>
       <c r="AC52" s="27" t="n">
-        <v>0.826923076923077</v>
+        <v>0.82692308</v>
       </c>
       <c r="AD52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AE52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AF52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AG52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AH52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AI52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AJ52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AK52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AL52" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19074,103 +19074,103 @@
         <v>1</v>
       </c>
       <c r="F53" s="27" t="n">
-        <v>0.976744186046512</v>
+        <v>0.97674419</v>
       </c>
       <c r="G53" s="27" t="n">
-        <v>0.976744186046512</v>
+        <v>0.97674419</v>
       </c>
       <c r="H53" s="27" t="n">
-        <v>0.976744186046512</v>
+        <v>0.97674419</v>
       </c>
       <c r="I53" s="27" t="n">
-        <v>0.976744186046512</v>
+        <v>0.97674419</v>
       </c>
       <c r="J53" s="27" t="n">
-        <v>0.976744186046512</v>
+        <v>0.97674419</v>
       </c>
       <c r="K53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="L53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="M53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="N53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="O53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="P53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="Q53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="R53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="S53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="T53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="U53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="V53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="W53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="X53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="Y53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="Z53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="AA53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="AB53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="AC53" s="27" t="n">
-        <v>0.953488372093023</v>
+        <v>0.95348837</v>
       </c>
       <c r="AD53" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AE53" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AF53" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AG53" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AH53" s="27" t="n">
-        <v>0.906976744186046</v>
+        <v>0.90697674</v>
       </c>
       <c r="AI53" s="27" t="n">
-        <v>0.883720930232558</v>
+        <v>0.88372093</v>
       </c>
       <c r="AJ53" s="27" t="n">
-        <v>0.86046511627907</v>
+        <v>0.86046512</v>
       </c>
       <c r="AK53" s="27" t="n">
-        <v>0.813953488372093</v>
+        <v>0.81395349</v>
       </c>
       <c r="AL53" s="27" t="n">
-        <v>0.813953488372093</v>
+        <v>0.81395349</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19184,109 +19184,109 @@
         <v>1</v>
       </c>
       <c r="D54" s="27" t="n">
-        <v>0.980769230769231</v>
+        <v>0.98076923</v>
       </c>
       <c r="E54" s="27" t="n">
-        <v>0.980769230769231</v>
+        <v>0.98076923</v>
       </c>
       <c r="F54" s="27" t="n">
-        <v>0.980769230769231</v>
+        <v>0.98076923</v>
       </c>
       <c r="G54" s="27" t="n">
-        <v>0.980769230769231</v>
+        <v>0.98076923</v>
       </c>
       <c r="H54" s="27" t="n">
-        <v>0.961538461538462</v>
+        <v>0.96153846</v>
       </c>
       <c r="I54" s="27" t="n">
-        <v>0.961538461538462</v>
+        <v>0.96153846</v>
       </c>
       <c r="J54" s="27" t="n">
-        <v>0.961538461538462</v>
+        <v>0.96153846</v>
       </c>
       <c r="K54" s="27" t="n">
-        <v>0.942307692307692</v>
+        <v>0.94230769</v>
       </c>
       <c r="L54" s="27" t="n">
-        <v>0.942307692307692</v>
+        <v>0.94230769</v>
       </c>
       <c r="M54" s="27" t="n">
-        <v>0.942307692307692</v>
+        <v>0.94230769</v>
       </c>
       <c r="N54" s="27" t="n">
-        <v>0.942307692307692</v>
+        <v>0.94230769</v>
       </c>
       <c r="O54" s="27" t="n">
-        <v>0.923076923076923</v>
+        <v>0.92307692</v>
       </c>
       <c r="P54" s="27" t="n">
-        <v>0.903846153846154</v>
+        <v>0.90384615</v>
       </c>
       <c r="Q54" s="27" t="n">
-        <v>0.884615384615385</v>
+        <v>0.88461538</v>
       </c>
       <c r="R54" s="27" t="n">
-        <v>0.884615384615385</v>
+        <v>0.88461538</v>
       </c>
       <c r="S54" s="27" t="n">
-        <v>0.884615384615385</v>
+        <v>0.88461538</v>
       </c>
       <c r="T54" s="27" t="n">
-        <v>0.884615384615385</v>
+        <v>0.88461538</v>
       </c>
       <c r="U54" s="27" t="n">
-        <v>0.865384615384615</v>
+        <v>0.86538462</v>
       </c>
       <c r="V54" s="27" t="n">
-        <v>0.865384615384615</v>
+        <v>0.86538462</v>
       </c>
       <c r="W54" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="X54" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="Y54" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="Z54" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AA54" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="AB54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AC54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AD54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AE54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AF54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AG54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AH54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AI54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AJ54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AK54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
       <c r="AL54" s="27" t="n">
-        <v>0.788461538461538</v>
+        <v>0.78846154</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19300,109 +19300,109 @@
         <v>1</v>
       </c>
       <c r="D55" s="27" t="n">
-        <v>0.985074626865672</v>
+        <v>0.98507463</v>
       </c>
       <c r="E55" s="27" t="n">
-        <v>0.985074626865672</v>
+        <v>0.98507463</v>
       </c>
       <c r="F55" s="27" t="n">
-        <v>0.985074626865672</v>
+        <v>0.98507463</v>
       </c>
       <c r="G55" s="27" t="n">
-        <v>0.970149253731343</v>
+        <v>0.97014925</v>
       </c>
       <c r="H55" s="27" t="n">
-        <v>0.970149253731343</v>
+        <v>0.97014925</v>
       </c>
       <c r="I55" s="27" t="n">
-        <v>0.970149253731343</v>
+        <v>0.97014925</v>
       </c>
       <c r="J55" s="27" t="n">
-        <v>0.970149253731343</v>
+        <v>0.97014925</v>
       </c>
       <c r="K55" s="27" t="n">
-        <v>0.970149253731343</v>
+        <v>0.97014925</v>
       </c>
       <c r="L55" s="27" t="n">
-        <v>0.955223880597015</v>
+        <v>0.95522388</v>
       </c>
       <c r="M55" s="27" t="n">
-        <v>0.955223880597015</v>
+        <v>0.95522388</v>
       </c>
       <c r="N55" s="27" t="n">
-        <v>0.955223880597015</v>
+        <v>0.95522388</v>
       </c>
       <c r="O55" s="27" t="n">
-        <v>0.940298507462687</v>
+        <v>0.94029851</v>
       </c>
       <c r="P55" s="27" t="n">
-        <v>0.940298507462687</v>
+        <v>0.94029851</v>
       </c>
       <c r="Q55" s="27" t="n">
-        <v>0.940298507462687</v>
+        <v>0.94029851</v>
       </c>
       <c r="R55" s="27" t="n">
-        <v>0.940298507462687</v>
+        <v>0.94029851</v>
       </c>
       <c r="S55" s="27" t="n">
-        <v>0.940298507462687</v>
+        <v>0.94029851</v>
       </c>
       <c r="T55" s="27" t="n">
-        <v>0.940298507462687</v>
+        <v>0.94029851</v>
       </c>
       <c r="U55" s="27" t="n">
-        <v>0.940298507462687</v>
+        <v>0.94029851</v>
       </c>
       <c r="V55" s="27" t="n">
-        <v>0.940298507462687</v>
+        <v>0.94029851</v>
       </c>
       <c r="W55" s="27" t="n">
-        <v>0.925373134328358</v>
+        <v>0.92537313</v>
       </c>
       <c r="X55" s="27" t="n">
-        <v>0.925373134328358</v>
+        <v>0.92537313</v>
       </c>
       <c r="Y55" s="27" t="n">
-        <v>0.925373134328358</v>
+        <v>0.92537313</v>
       </c>
       <c r="Z55" s="27" t="n">
-        <v>0.925373134328358</v>
+        <v>0.92537313</v>
       </c>
       <c r="AA55" s="27" t="n">
-        <v>0.895522388059702</v>
+        <v>0.89552239</v>
       </c>
       <c r="AB55" s="27" t="n">
-        <v>0.880597014925373</v>
+        <v>0.88059701</v>
       </c>
       <c r="AC55" s="27" t="n">
-        <v>0.865671641791045</v>
+        <v>0.86567164</v>
       </c>
       <c r="AD55" s="27" t="n">
-        <v>0.865671641791045</v>
+        <v>0.86567164</v>
       </c>
       <c r="AE55" s="27" t="n">
-        <v>0.82089552238806</v>
+        <v>0.82089552</v>
       </c>
       <c r="AF55" s="27" t="n">
-        <v>0.805970149253731</v>
+        <v>0.80597015</v>
       </c>
       <c r="AG55" s="27" t="n">
-        <v>0.761194029850746</v>
+        <v>0.76119403</v>
       </c>
       <c r="AH55" s="27" t="n">
-        <v>0.746268656716418</v>
+        <v>0.74626866</v>
       </c>
       <c r="AI55" s="27" t="n">
-        <v>0.746268656716418</v>
+        <v>0.74626866</v>
       </c>
       <c r="AJ55" s="27" t="n">
-        <v>0.746268656716418</v>
+        <v>0.74626866</v>
       </c>
       <c r="AK55" s="27" t="n">
-        <v>0.73134328358209</v>
+        <v>0.73134328</v>
       </c>
       <c r="AL55" s="27" t="n">
-        <v>0.73134328358209</v>
+        <v>0.73134328</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19416,61 +19416,61 @@
         <v>1</v>
       </c>
       <c r="D56" s="27" t="n">
-        <v>0.983333333333333</v>
+        <v>0.98333333</v>
       </c>
       <c r="E56" s="27" t="n">
-        <v>0.983333333333333</v>
+        <v>0.98333333</v>
       </c>
       <c r="F56" s="27" t="n">
-        <v>0.966666666666667</v>
+        <v>0.96666667</v>
       </c>
       <c r="G56" s="27" t="n">
-        <v>0.933333333333333</v>
+        <v>0.93333333</v>
       </c>
       <c r="H56" s="27" t="n">
-        <v>0.933333333333333</v>
+        <v>0.93333333</v>
       </c>
       <c r="I56" s="27" t="n">
-        <v>0.933333333333333</v>
+        <v>0.93333333</v>
       </c>
       <c r="J56" s="27" t="n">
-        <v>0.933333333333333</v>
+        <v>0.93333333</v>
       </c>
       <c r="K56" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="L56" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="M56" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="N56" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="O56" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="P56" s="27" t="n">
-        <v>0.866666666666667</v>
+        <v>0.86666667</v>
       </c>
       <c r="Q56" s="27" t="n">
-        <v>0.866666666666667</v>
+        <v>0.86666667</v>
       </c>
       <c r="R56" s="27" t="n">
         <v>0.85</v>
       </c>
       <c r="S56" s="27" t="n">
-        <v>0.833333333333334</v>
+        <v>0.83333333</v>
       </c>
       <c r="T56" s="27" t="n">
-        <v>0.833333333333334</v>
+        <v>0.83333333</v>
       </c>
       <c r="U56" s="27" t="n">
-        <v>0.783333333333333</v>
+        <v>0.78333333</v>
       </c>
       <c r="V56" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="W56" s="27" t="n">
         <v>0.75</v>
@@ -19482,43 +19482,43 @@
         <v>0.75</v>
       </c>
       <c r="Z56" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
       <c r="AA56" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
       <c r="AB56" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
       <c r="AC56" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
       <c r="AD56" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
       <c r="AE56" s="27" t="n">
-        <v>0.716666666666667</v>
+        <v>0.71666667</v>
       </c>
       <c r="AF56" s="27" t="n">
         <v>0.7</v>
       </c>
       <c r="AG56" s="27" t="n">
-        <v>0.683333333333333</v>
+        <v>0.68333333</v>
       </c>
       <c r="AH56" s="27" t="n">
-        <v>0.683333333333333</v>
+        <v>0.68333333</v>
       </c>
       <c r="AI56" s="27" t="n">
-        <v>0.683333333333333</v>
+        <v>0.68333333</v>
       </c>
       <c r="AJ56" s="27" t="n">
-        <v>0.666666666666667</v>
+        <v>0.66666667</v>
       </c>
       <c r="AK56" s="27" t="n">
-        <v>0.666666666666667</v>
+        <v>0.66666667</v>
       </c>
       <c r="AL56" s="27" t="n">
-        <v>0.666666666666667</v>
+        <v>0.66666667</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19538,103 +19538,103 @@
         <v>1</v>
       </c>
       <c r="F57" s="27" t="n">
-        <v>0.975609756097561</v>
+        <v>0.97560976</v>
       </c>
       <c r="G57" s="27" t="n">
-        <v>0.975609756097561</v>
+        <v>0.97560976</v>
       </c>
       <c r="H57" s="27" t="n">
-        <v>0.975609756097561</v>
+        <v>0.97560976</v>
       </c>
       <c r="I57" s="27" t="n">
-        <v>0.951219512195122</v>
+        <v>0.95121951</v>
       </c>
       <c r="J57" s="27" t="n">
-        <v>0.951219512195122</v>
+        <v>0.95121951</v>
       </c>
       <c r="K57" s="27" t="n">
-        <v>0.951219512195122</v>
+        <v>0.95121951</v>
       </c>
       <c r="L57" s="27" t="n">
-        <v>0.926829268292683</v>
+        <v>0.92682927</v>
       </c>
       <c r="M57" s="27" t="n">
-        <v>0.926829268292683</v>
+        <v>0.92682927</v>
       </c>
       <c r="N57" s="27" t="n">
-        <v>0.926829268292683</v>
+        <v>0.92682927</v>
       </c>
       <c r="O57" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="P57" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="Q57" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="R57" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="S57" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="T57" s="27" t="n">
-        <v>0.878048780487805</v>
+        <v>0.87804878</v>
       </c>
       <c r="U57" s="27" t="n">
-        <v>0.878048780487805</v>
+        <v>0.87804878</v>
       </c>
       <c r="V57" s="27" t="n">
-        <v>0.853658536585366</v>
+        <v>0.85365854</v>
       </c>
       <c r="W57" s="27" t="n">
-        <v>0.853658536585366</v>
+        <v>0.85365854</v>
       </c>
       <c r="X57" s="27" t="n">
-        <v>0.853658536585366</v>
+        <v>0.85365854</v>
       </c>
       <c r="Y57" s="27" t="n">
-        <v>0.853658536585366</v>
+        <v>0.85365854</v>
       </c>
       <c r="Z57" s="27" t="n">
-        <v>0.829268292682927</v>
+        <v>0.82926829</v>
       </c>
       <c r="AA57" s="27" t="n">
-        <v>0.804878048780488</v>
+        <v>0.80487805</v>
       </c>
       <c r="AB57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AC57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AD57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AE57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AF57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AG57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AH57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AI57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AJ57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AK57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="AL57" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19764,109 +19764,109 @@
         <v>1</v>
       </c>
       <c r="D59" s="27" t="n">
-        <v>0.982758620689655</v>
+        <v>0.98275862</v>
       </c>
       <c r="E59" s="27" t="n">
-        <v>0.982758620689655</v>
+        <v>0.98275862</v>
       </c>
       <c r="F59" s="27" t="n">
-        <v>0.982758620689655</v>
+        <v>0.98275862</v>
       </c>
       <c r="G59" s="27" t="n">
-        <v>0.982758620689655</v>
+        <v>0.98275862</v>
       </c>
       <c r="H59" s="27" t="n">
-        <v>0.965517241379311</v>
+        <v>0.96551724</v>
       </c>
       <c r="I59" s="27" t="n">
-        <v>0.948275862068966</v>
+        <v>0.94827586</v>
       </c>
       <c r="J59" s="27" t="n">
-        <v>0.913793103448276</v>
+        <v>0.9137931</v>
       </c>
       <c r="K59" s="27" t="n">
-        <v>0.896551724137931</v>
+        <v>0.89655172</v>
       </c>
       <c r="L59" s="27" t="n">
-        <v>0.896551724137931</v>
+        <v>0.89655172</v>
       </c>
       <c r="M59" s="27" t="n">
-        <v>0.879310344827586</v>
+        <v>0.87931034</v>
       </c>
       <c r="N59" s="27" t="n">
-        <v>0.879310344827586</v>
+        <v>0.87931034</v>
       </c>
       <c r="O59" s="27" t="n">
-        <v>0.862068965517241</v>
+        <v>0.86206897</v>
       </c>
       <c r="P59" s="27" t="n">
-        <v>0.862068965517241</v>
+        <v>0.86206897</v>
       </c>
       <c r="Q59" s="27" t="n">
-        <v>0.862068965517241</v>
+        <v>0.86206897</v>
       </c>
       <c r="R59" s="27" t="n">
-        <v>0.844827586206897</v>
+        <v>0.84482759</v>
       </c>
       <c r="S59" s="27" t="n">
-        <v>0.844827586206897</v>
+        <v>0.84482759</v>
       </c>
       <c r="T59" s="27" t="n">
-        <v>0.844827586206897</v>
+        <v>0.84482759</v>
       </c>
       <c r="U59" s="27" t="n">
-        <v>0.827586206896552</v>
+        <v>0.82758621</v>
       </c>
       <c r="V59" s="27" t="n">
-        <v>0.827586206896552</v>
+        <v>0.82758621</v>
       </c>
       <c r="W59" s="27" t="n">
-        <v>0.827586206896552</v>
+        <v>0.82758621</v>
       </c>
       <c r="X59" s="27" t="n">
-        <v>0.827586206896552</v>
+        <v>0.82758621</v>
       </c>
       <c r="Y59" s="27" t="n">
-        <v>0.810344827586207</v>
+        <v>0.81034483</v>
       </c>
       <c r="Z59" s="27" t="n">
-        <v>0.810344827586207</v>
+        <v>0.81034483</v>
       </c>
       <c r="AA59" s="27" t="n">
-        <v>0.810344827586207</v>
+        <v>0.81034483</v>
       </c>
       <c r="AB59" s="27" t="n">
-        <v>0.810344827586207</v>
+        <v>0.81034483</v>
       </c>
       <c r="AC59" s="27" t="n">
-        <v>0.810344827586207</v>
+        <v>0.81034483</v>
       </c>
       <c r="AD59" s="27" t="n">
-        <v>0.793103448275862</v>
+        <v>0.79310345</v>
       </c>
       <c r="AE59" s="27" t="n">
-        <v>0.793103448275862</v>
+        <v>0.79310345</v>
       </c>
       <c r="AF59" s="27" t="n">
-        <v>0.775862068965517</v>
+        <v>0.77586207</v>
       </c>
       <c r="AG59" s="27" t="n">
-        <v>0.775862068965517</v>
+        <v>0.77586207</v>
       </c>
       <c r="AH59" s="27" t="n">
-        <v>0.775862068965517</v>
+        <v>0.77586207</v>
       </c>
       <c r="AI59" s="27" t="n">
-        <v>0.775862068965517</v>
+        <v>0.77586207</v>
       </c>
       <c r="AJ59" s="27" t="n">
-        <v>0.775862068965517</v>
+        <v>0.77586207</v>
       </c>
       <c r="AK59" s="27" t="n">
-        <v>0.741379310344828</v>
+        <v>0.74137931</v>
       </c>
       <c r="AL59" s="27" t="n">
-        <v>0.741379310344828</v>
+        <v>0.74137931</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19889,100 +19889,100 @@
         <v>1</v>
       </c>
       <c r="G60" s="27" t="n">
-        <v>0.982456140350877</v>
+        <v>0.98245614</v>
       </c>
       <c r="H60" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="I60" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="J60" s="27" t="n">
-        <v>0.947368421052632</v>
+        <v>0.94736842</v>
       </c>
       <c r="K60" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="L60" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="M60" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="N60" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="O60" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="P60" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="Q60" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="R60" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="S60" s="27" t="n">
-        <v>0.912280701754386</v>
+        <v>0.9122807</v>
       </c>
       <c r="T60" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="U60" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="V60" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="W60" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="X60" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="Y60" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="Z60" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="AA60" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="AB60" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="AC60" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="AD60" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="AE60" s="27" t="n">
-        <v>0.842105263157895</v>
+        <v>0.84210526</v>
       </c>
       <c r="AF60" s="27" t="n">
-        <v>0.842105263157895</v>
+        <v>0.84210526</v>
       </c>
       <c r="AG60" s="27" t="n">
-        <v>0.842105263157895</v>
+        <v>0.84210526</v>
       </c>
       <c r="AH60" s="27" t="n">
-        <v>0.842105263157895</v>
+        <v>0.84210526</v>
       </c>
       <c r="AI60" s="27" t="n">
-        <v>0.824561403508772</v>
+        <v>0.8245614</v>
       </c>
       <c r="AJ60" s="27" t="n">
-        <v>0.824561403508772</v>
+        <v>0.8245614</v>
       </c>
       <c r="AK60" s="27" t="n">
-        <v>0.807017543859649</v>
+        <v>0.80701754</v>
       </c>
       <c r="AL60" s="27" t="n">
-        <v>0.807017543859649</v>
+        <v>0.80701754</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20014,91 +20014,91 @@
         <v>1</v>
       </c>
       <c r="J61" s="27" t="n">
-        <v>0.982456140350877</v>
+        <v>0.98245614</v>
       </c>
       <c r="K61" s="27" t="n">
-        <v>0.964912280701754</v>
+        <v>0.96491228</v>
       </c>
       <c r="L61" s="27" t="n">
-        <v>0.929824561403509</v>
+        <v>0.92982456</v>
       </c>
       <c r="M61" s="27" t="n">
-        <v>0.912280701754386</v>
+        <v>0.9122807</v>
       </c>
       <c r="N61" s="27" t="n">
-        <v>0.912280701754386</v>
+        <v>0.9122807</v>
       </c>
       <c r="O61" s="27" t="n">
-        <v>0.912280701754386</v>
+        <v>0.9122807</v>
       </c>
       <c r="P61" s="27" t="n">
-        <v>0.894736842105263</v>
+        <v>0.89473684</v>
       </c>
       <c r="Q61" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="R61" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="S61" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="T61" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="U61" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="V61" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="W61" s="27" t="n">
-        <v>0.87719298245614</v>
+        <v>0.87719298</v>
       </c>
       <c r="X61" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="Y61" s="27" t="n">
-        <v>0.859649122807018</v>
+        <v>0.85964912</v>
       </c>
       <c r="Z61" s="27" t="n">
-        <v>0.842105263157895</v>
+        <v>0.84210526</v>
       </c>
       <c r="AA61" s="27" t="n">
-        <v>0.824561403508772</v>
+        <v>0.8245614</v>
       </c>
       <c r="AB61" s="27" t="n">
-        <v>0.824561403508772</v>
+        <v>0.8245614</v>
       </c>
       <c r="AC61" s="27" t="n">
-        <v>0.807017543859649</v>
+        <v>0.80701754</v>
       </c>
       <c r="AD61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
       <c r="AE61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
       <c r="AF61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
       <c r="AG61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
       <c r="AH61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
       <c r="AI61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
       <c r="AJ61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
       <c r="AK61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
       <c r="AL61" s="27" t="n">
-        <v>0.771929824561404</v>
+        <v>0.77192982</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20118,103 +20118,103 @@
         <v>1</v>
       </c>
       <c r="F62" s="27" t="n">
-        <v>0.984126984126984</v>
+        <v>0.98412698</v>
       </c>
       <c r="G62" s="27" t="n">
-        <v>0.984126984126984</v>
+        <v>0.98412698</v>
       </c>
       <c r="H62" s="27" t="n">
-        <v>0.968253968253968</v>
+        <v>0.96825397</v>
       </c>
       <c r="I62" s="27" t="n">
-        <v>0.968253968253968</v>
+        <v>0.96825397</v>
       </c>
       <c r="J62" s="27" t="n">
-        <v>0.936507936507936</v>
+        <v>0.93650794</v>
       </c>
       <c r="K62" s="27" t="n">
-        <v>0.936507936507936</v>
+        <v>0.93650794</v>
       </c>
       <c r="L62" s="27" t="n">
-        <v>0.936507936507936</v>
+        <v>0.93650794</v>
       </c>
       <c r="M62" s="27" t="n">
-        <v>0.920634920634921</v>
+        <v>0.92063492</v>
       </c>
       <c r="N62" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="O62" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="P62" s="27" t="n">
-        <v>0.888888888888889</v>
+        <v>0.88888889</v>
       </c>
       <c r="Q62" s="27" t="n">
-        <v>0.857142857142857</v>
+        <v>0.85714286</v>
       </c>
       <c r="R62" s="27" t="n">
-        <v>0.857142857142857</v>
+        <v>0.85714286</v>
       </c>
       <c r="S62" s="27" t="n">
-        <v>0.841269841269841</v>
+        <v>0.84126984</v>
       </c>
       <c r="T62" s="27" t="n">
-        <v>0.841269841269841</v>
+        <v>0.84126984</v>
       </c>
       <c r="U62" s="27" t="n">
-        <v>0.841269841269841</v>
+        <v>0.84126984</v>
       </c>
       <c r="V62" s="27" t="n">
-        <v>0.80952380952381</v>
+        <v>0.80952381</v>
       </c>
       <c r="W62" s="27" t="n">
-        <v>0.80952380952381</v>
+        <v>0.80952381</v>
       </c>
       <c r="X62" s="27" t="n">
-        <v>0.793650793650794</v>
+        <v>0.79365079</v>
       </c>
       <c r="Y62" s="27" t="n">
-        <v>0.793650793650794</v>
+        <v>0.79365079</v>
       </c>
       <c r="Z62" s="27" t="n">
-        <v>0.777777777777778</v>
+        <v>0.77777778</v>
       </c>
       <c r="AA62" s="27" t="n">
-        <v>0.761904761904762</v>
+        <v>0.76190476</v>
       </c>
       <c r="AB62" s="27" t="n">
-        <v>0.761904761904762</v>
+        <v>0.76190476</v>
       </c>
       <c r="AC62" s="27" t="n">
-        <v>0.761904761904762</v>
+        <v>0.76190476</v>
       </c>
       <c r="AD62" s="27" t="n">
-        <v>0.761904761904762</v>
+        <v>0.76190476</v>
       </c>
       <c r="AE62" s="27" t="n">
-        <v>0.73015873015873</v>
+        <v>0.73015873</v>
       </c>
       <c r="AF62" s="27" t="n">
-        <v>0.73015873015873</v>
+        <v>0.73015873</v>
       </c>
       <c r="AG62" s="27" t="n">
-        <v>0.73015873015873</v>
+        <v>0.73015873</v>
       </c>
       <c r="AH62" s="27" t="n">
-        <v>0.73015873015873</v>
+        <v>0.73015873</v>
       </c>
       <c r="AI62" s="27" t="n">
-        <v>0.73015873015873</v>
+        <v>0.73015873</v>
       </c>
       <c r="AJ62" s="27" t="n">
-        <v>0.714285714285714</v>
+        <v>0.71428571</v>
       </c>
       <c r="AK62" s="27" t="n">
-        <v>0.714285714285714</v>
+        <v>0.71428571</v>
       </c>
       <c r="AL62" s="27" t="n">
-        <v>0.714285714285714</v>
+        <v>0.71428571</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20237,100 +20237,100 @@
         <v>1</v>
       </c>
       <c r="G63" s="27" t="n">
-        <v>0.984615384615385</v>
+        <v>0.98461538</v>
       </c>
       <c r="H63" s="27" t="n">
-        <v>0.969230769230769</v>
+        <v>0.96923077</v>
       </c>
       <c r="I63" s="27" t="n">
-        <v>0.969230769230769</v>
+        <v>0.96923077</v>
       </c>
       <c r="J63" s="27" t="n">
-        <v>0.953846153846154</v>
+        <v>0.95384615</v>
       </c>
       <c r="K63" s="27" t="n">
-        <v>0.923076923076923</v>
+        <v>0.92307692</v>
       </c>
       <c r="L63" s="27" t="n">
-        <v>0.907692307692308</v>
+        <v>0.90769231</v>
       </c>
       <c r="M63" s="27" t="n">
-        <v>0.907692307692308</v>
+        <v>0.90769231</v>
       </c>
       <c r="N63" s="27" t="n">
-        <v>0.907692307692308</v>
+        <v>0.90769231</v>
       </c>
       <c r="O63" s="27" t="n">
-        <v>0.907692307692308</v>
+        <v>0.90769231</v>
       </c>
       <c r="P63" s="27" t="n">
-        <v>0.907692307692308</v>
+        <v>0.90769231</v>
       </c>
       <c r="Q63" s="27" t="n">
-        <v>0.907692307692308</v>
+        <v>0.90769231</v>
       </c>
       <c r="R63" s="27" t="n">
-        <v>0.892307692307692</v>
+        <v>0.89230769</v>
       </c>
       <c r="S63" s="27" t="n">
-        <v>0.876923076923077</v>
+        <v>0.87692308</v>
       </c>
       <c r="T63" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="U63" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="V63" s="27" t="n">
-        <v>0.815384615384615</v>
+        <v>0.81538462</v>
       </c>
       <c r="W63" s="27" t="n">
-        <v>0.815384615384615</v>
+        <v>0.81538462</v>
       </c>
       <c r="X63" s="27" t="n">
-        <v>0.815384615384615</v>
+        <v>0.81538462</v>
       </c>
       <c r="Y63" s="27" t="n">
-        <v>0.784615384615385</v>
+        <v>0.78461538</v>
       </c>
       <c r="Z63" s="27" t="n">
-        <v>0.769230769230769</v>
+        <v>0.76923077</v>
       </c>
       <c r="AA63" s="27" t="n">
-        <v>0.753846153846154</v>
+        <v>0.75384615</v>
       </c>
       <c r="AB63" s="27" t="n">
-        <v>0.738461538461539</v>
+        <v>0.73846154</v>
       </c>
       <c r="AC63" s="27" t="n">
-        <v>0.738461538461539</v>
+        <v>0.73846154</v>
       </c>
       <c r="AD63" s="27" t="n">
-        <v>0.738461538461539</v>
+        <v>0.73846154</v>
       </c>
       <c r="AE63" s="27" t="n">
-        <v>0.723076923076923</v>
+        <v>0.72307692</v>
       </c>
       <c r="AF63" s="27" t="n">
-        <v>0.692307692307692</v>
+        <v>0.69230769</v>
       </c>
       <c r="AG63" s="27" t="n">
-        <v>0.661538461538461</v>
+        <v>0.66153846</v>
       </c>
       <c r="AH63" s="27" t="n">
-        <v>0.646153846153846</v>
+        <v>0.64615385</v>
       </c>
       <c r="AI63" s="27" t="n">
-        <v>0.646153846153846</v>
+        <v>0.64615385</v>
       </c>
       <c r="AJ63" s="27" t="n">
-        <v>0.646153846153846</v>
+        <v>0.64615385</v>
       </c>
       <c r="AK63" s="27" t="n">
-        <v>0.630769230769231</v>
+        <v>0.63076923</v>
       </c>
       <c r="AL63" s="27" t="n">
-        <v>0.630769230769231</v>
+        <v>0.63076923</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20347,106 +20347,106 @@
         <v>1</v>
       </c>
       <c r="E64" s="27" t="n">
-        <v>0.983606557377049</v>
+        <v>0.98360656</v>
       </c>
       <c r="F64" s="27" t="n">
-        <v>0.983606557377049</v>
+        <v>0.98360656</v>
       </c>
       <c r="G64" s="27" t="n">
-        <v>0.967213114754098</v>
+        <v>0.96721311</v>
       </c>
       <c r="H64" s="27" t="n">
-        <v>0.934426229508197</v>
+        <v>0.93442623</v>
       </c>
       <c r="I64" s="27" t="n">
-        <v>0.918032786885246</v>
+        <v>0.91803279</v>
       </c>
       <c r="J64" s="27" t="n">
-        <v>0.918032786885246</v>
+        <v>0.91803279</v>
       </c>
       <c r="K64" s="27" t="n">
-        <v>0.918032786885246</v>
+        <v>0.91803279</v>
       </c>
       <c r="L64" s="27" t="n">
-        <v>0.918032786885246</v>
+        <v>0.91803279</v>
       </c>
       <c r="M64" s="27" t="n">
-        <v>0.918032786885246</v>
+        <v>0.91803279</v>
       </c>
       <c r="N64" s="27" t="n">
-        <v>0.918032786885246</v>
+        <v>0.91803279</v>
       </c>
       <c r="O64" s="27" t="n">
-        <v>0.918032786885246</v>
+        <v>0.91803279</v>
       </c>
       <c r="P64" s="27" t="n">
-        <v>0.885245901639344</v>
+        <v>0.8852459</v>
       </c>
       <c r="Q64" s="27" t="n">
-        <v>0.868852459016393</v>
+        <v>0.86885246</v>
       </c>
       <c r="R64" s="27" t="n">
-        <v>0.852459016393443</v>
+        <v>0.85245902</v>
       </c>
       <c r="S64" s="27" t="n">
-        <v>0.852459016393443</v>
+        <v>0.85245902</v>
       </c>
       <c r="T64" s="27" t="n">
-        <v>0.852459016393443</v>
+        <v>0.85245902</v>
       </c>
       <c r="U64" s="27" t="n">
-        <v>0.836065573770492</v>
+        <v>0.83606557</v>
       </c>
       <c r="V64" s="27" t="n">
-        <v>0.836065573770492</v>
+        <v>0.83606557</v>
       </c>
       <c r="W64" s="27" t="n">
-        <v>0.819672131147541</v>
+        <v>0.81967213</v>
       </c>
       <c r="X64" s="27" t="n">
-        <v>0.786885245901639</v>
+        <v>0.78688525</v>
       </c>
       <c r="Y64" s="27" t="n">
-        <v>0.786885245901639</v>
+        <v>0.78688525</v>
       </c>
       <c r="Z64" s="27" t="n">
-        <v>0.754098360655738</v>
+        <v>0.75409836</v>
       </c>
       <c r="AA64" s="27" t="n">
-        <v>0.737704918032787</v>
+        <v>0.73770492</v>
       </c>
       <c r="AB64" s="27" t="n">
-        <v>0.737704918032787</v>
+        <v>0.73770492</v>
       </c>
       <c r="AC64" s="27" t="n">
-        <v>0.737704918032787</v>
+        <v>0.73770492</v>
       </c>
       <c r="AD64" s="27" t="n">
-        <v>0.721311475409836</v>
+        <v>0.72131148</v>
       </c>
       <c r="AE64" s="27" t="n">
-        <v>0.721311475409836</v>
+        <v>0.72131148</v>
       </c>
       <c r="AF64" s="27" t="n">
-        <v>0.721311475409836</v>
+        <v>0.72131148</v>
       </c>
       <c r="AG64" s="27" t="n">
-        <v>0.721311475409836</v>
+        <v>0.72131148</v>
       </c>
       <c r="AH64" s="27" t="n">
-        <v>0.704918032786885</v>
+        <v>0.70491803</v>
       </c>
       <c r="AI64" s="27" t="n">
-        <v>0.704918032786885</v>
+        <v>0.70491803</v>
       </c>
       <c r="AJ64" s="27" t="n">
-        <v>0.704918032786885</v>
+        <v>0.70491803</v>
       </c>
       <c r="AK64" s="27" t="n">
-        <v>0.704918032786885</v>
+        <v>0.70491803</v>
       </c>
       <c r="AL64" s="27" t="n">
-        <v>0.704918032786885</v>
+        <v>0.70491803</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20472,97 +20472,97 @@
         <v>1</v>
       </c>
       <c r="H65" s="27" t="n">
-        <v>0.980769230769231</v>
+        <v>0.98076923</v>
       </c>
       <c r="I65" s="27" t="n">
-        <v>0.961538461538462</v>
+        <v>0.96153846</v>
       </c>
       <c r="J65" s="27" t="n">
-        <v>0.942307692307692</v>
+        <v>0.94230769</v>
       </c>
       <c r="K65" s="27" t="n">
-        <v>0.942307692307692</v>
+        <v>0.94230769</v>
       </c>
       <c r="L65" s="27" t="n">
-        <v>0.923076923076923</v>
+        <v>0.92307692</v>
       </c>
       <c r="M65" s="27" t="n">
-        <v>0.923076923076923</v>
+        <v>0.92307692</v>
       </c>
       <c r="N65" s="27" t="n">
-        <v>0.903846153846154</v>
+        <v>0.90384615</v>
       </c>
       <c r="O65" s="27" t="n">
-        <v>0.903846153846154</v>
+        <v>0.90384615</v>
       </c>
       <c r="P65" s="27" t="n">
-        <v>0.903846153846154</v>
+        <v>0.90384615</v>
       </c>
       <c r="Q65" s="27" t="n">
-        <v>0.903846153846154</v>
+        <v>0.90384615</v>
       </c>
       <c r="R65" s="27" t="n">
-        <v>0.903846153846154</v>
+        <v>0.90384615</v>
       </c>
       <c r="S65" s="27" t="n">
-        <v>0.884615384615385</v>
+        <v>0.88461538</v>
       </c>
       <c r="T65" s="27" t="n">
-        <v>0.865384615384615</v>
+        <v>0.86538462</v>
       </c>
       <c r="U65" s="27" t="n">
-        <v>0.865384615384615</v>
+        <v>0.86538462</v>
       </c>
       <c r="V65" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="W65" s="27" t="n">
-        <v>0.846153846153846</v>
+        <v>0.84615385</v>
       </c>
       <c r="X65" s="27" t="n">
-        <v>0.826923076923077</v>
+        <v>0.82692308</v>
       </c>
       <c r="Y65" s="27" t="n">
-        <v>0.807692307692308</v>
+        <v>0.80769231</v>
       </c>
       <c r="Z65" s="27" t="n">
-        <v>0.769230769230769</v>
+        <v>0.76923077</v>
       </c>
       <c r="AA65" s="27" t="n">
-        <v>0.769230769230769</v>
+        <v>0.76923077</v>
       </c>
       <c r="AB65" s="27" t="n">
-        <v>0.769230769230769</v>
+        <v>0.76923077</v>
       </c>
       <c r="AC65" s="27" t="n">
-        <v>0.730769230769231</v>
+        <v>0.73076923</v>
       </c>
       <c r="AD65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
       <c r="AE65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
       <c r="AF65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
       <c r="AG65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
       <c r="AH65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
       <c r="AI65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
       <c r="AJ65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
       <c r="AK65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
       <c r="AL65" s="27" t="n">
-        <v>0.711538461538462</v>
+        <v>0.71153846</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20689,103 +20689,103 @@
         <v>1</v>
       </c>
       <c r="C67" s="27" t="n">
-        <v>0.988095238095238</v>
+        <v>0.98809524</v>
       </c>
       <c r="D67" s="27" t="n">
-        <v>0.988095238095238</v>
+        <v>0.98809524</v>
       </c>
       <c r="E67" s="27" t="n">
-        <v>0.988095238095238</v>
+        <v>0.98809524</v>
       </c>
       <c r="F67" s="27" t="n">
-        <v>0.976190476190476</v>
+        <v>0.97619048</v>
       </c>
       <c r="G67" s="27" t="n">
-        <v>0.952380952380952</v>
+        <v>0.95238095</v>
       </c>
       <c r="H67" s="27" t="n">
-        <v>0.904761904761905</v>
+        <v>0.9047619</v>
       </c>
       <c r="I67" s="27" t="n">
-        <v>0.904761904761905</v>
+        <v>0.9047619</v>
       </c>
       <c r="J67" s="27" t="n">
-        <v>0.857142857142857</v>
+        <v>0.85714286</v>
       </c>
       <c r="K67" s="27" t="n">
-        <v>0.857142857142857</v>
+        <v>0.85714286</v>
       </c>
       <c r="L67" s="27" t="n">
-        <v>0.833333333333334</v>
+        <v>0.83333333</v>
       </c>
       <c r="M67" s="27" t="n">
-        <v>0.80952380952381</v>
+        <v>0.80952381</v>
       </c>
       <c r="N67" s="27" t="n">
-        <v>0.797619047619048</v>
+        <v>0.79761905</v>
       </c>
       <c r="O67" s="27" t="n">
-        <v>0.773809523809524</v>
+        <v>0.77380952</v>
       </c>
       <c r="P67" s="27" t="n">
-        <v>0.761904761904762</v>
+        <v>0.76190476</v>
       </c>
       <c r="Q67" s="27" t="n">
         <v>0.75</v>
       </c>
       <c r="R67" s="27" t="n">
-        <v>0.738095238095238</v>
+        <v>0.73809524</v>
       </c>
       <c r="S67" s="27" t="n">
-        <v>0.738095238095238</v>
+        <v>0.73809524</v>
       </c>
       <c r="T67" s="27" t="n">
-        <v>0.702380952380952</v>
+        <v>0.70238095</v>
       </c>
       <c r="U67" s="27" t="n">
-        <v>0.678571428571429</v>
+        <v>0.67857143</v>
       </c>
       <c r="V67" s="27" t="n">
-        <v>0.654761904761905</v>
+        <v>0.6547619</v>
       </c>
       <c r="W67" s="27" t="n">
-        <v>0.642857142857143</v>
+        <v>0.64285714</v>
       </c>
       <c r="X67" s="27" t="n">
-        <v>0.630952380952381</v>
+        <v>0.63095238</v>
       </c>
       <c r="Y67" s="27" t="n">
-        <v>0.595238095238095</v>
+        <v>0.5952381</v>
       </c>
       <c r="Z67" s="27" t="n">
-        <v>0.595238095238095</v>
+        <v>0.5952381</v>
       </c>
       <c r="AA67" s="27" t="n">
-        <v>0.55952380952381</v>
+        <v>0.55952381</v>
       </c>
       <c r="AB67" s="27" t="n">
-        <v>0.547619047619048</v>
+        <v>0.54761905</v>
       </c>
       <c r="AC67" s="27" t="n">
-        <v>0.547619047619048</v>
+        <v>0.54761905</v>
       </c>
       <c r="AD67" s="27" t="n">
-        <v>0.547619047619048</v>
+        <v>0.54761905</v>
       </c>
       <c r="AE67" s="27" t="n">
-        <v>0.511904761904762</v>
+        <v>0.51190476</v>
       </c>
       <c r="AF67" s="27" t="n">
         <v>0.5</v>
       </c>
       <c r="AG67" s="27" t="n">
-        <v>0.476190476190476</v>
+        <v>0.47619048</v>
       </c>
       <c r="AH67" s="27" t="n">
-        <v>0.476190476190476</v>
+        <v>0.47619048</v>
       </c>
       <c r="AI67" s="27" t="n">
-        <v>0.464285714285714</v>
+        <v>0.46428571</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20805,85 +20805,85 @@
         <v>1</v>
       </c>
       <c r="F68" s="27" t="n">
-        <v>0.964285714285714</v>
+        <v>0.96428571</v>
       </c>
       <c r="G68" s="27" t="n">
-        <v>0.964285714285714</v>
+        <v>0.96428571</v>
       </c>
       <c r="H68" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="I68" s="27" t="n">
-        <v>0.880952380952381</v>
+        <v>0.88095238</v>
       </c>
       <c r="J68" s="27" t="n">
-        <v>0.880952380952381</v>
+        <v>0.88095238</v>
       </c>
       <c r="K68" s="27" t="n">
-        <v>0.880952380952381</v>
+        <v>0.88095238</v>
       </c>
       <c r="L68" s="27" t="n">
-        <v>0.845238095238095</v>
+        <v>0.8452381</v>
       </c>
       <c r="M68" s="27" t="n">
-        <v>0.821428571428571</v>
+        <v>0.82142857</v>
       </c>
       <c r="N68" s="27" t="n">
-        <v>0.797619047619048</v>
+        <v>0.79761905</v>
       </c>
       <c r="O68" s="27" t="n">
-        <v>0.785714285714286</v>
+        <v>0.78571429</v>
       </c>
       <c r="P68" s="27" t="n">
-        <v>0.761904761904762</v>
+        <v>0.76190476</v>
       </c>
       <c r="Q68" s="27" t="n">
-        <v>0.761904761904762</v>
+        <v>0.76190476</v>
       </c>
       <c r="R68" s="27" t="n">
-        <v>0.726190476190476</v>
+        <v>0.72619048</v>
       </c>
       <c r="S68" s="27" t="n">
-        <v>0.726190476190476</v>
+        <v>0.72619048</v>
       </c>
       <c r="T68" s="27" t="n">
-        <v>0.714285714285714</v>
+        <v>0.71428571</v>
       </c>
       <c r="U68" s="27" t="n">
-        <v>0.690476190476191</v>
+        <v>0.69047619</v>
       </c>
       <c r="V68" s="27" t="n">
-        <v>0.678571428571429</v>
+        <v>0.67857143</v>
       </c>
       <c r="W68" s="27" t="n">
-        <v>0.678571428571429</v>
+        <v>0.67857143</v>
       </c>
       <c r="X68" s="27" t="n">
-        <v>0.678571428571429</v>
+        <v>0.67857143</v>
       </c>
       <c r="Y68" s="27" t="n">
-        <v>0.678571428571429</v>
+        <v>0.67857143</v>
       </c>
       <c r="Z68" s="27" t="n">
-        <v>0.654761904761905</v>
+        <v>0.6547619</v>
       </c>
       <c r="AA68" s="27" t="n">
-        <v>0.642857142857143</v>
+        <v>0.64285714</v>
       </c>
       <c r="AB68" s="27" t="n">
-        <v>0.642857142857143</v>
+        <v>0.64285714</v>
       </c>
       <c r="AC68" s="27" t="n">
-        <v>0.630952380952381</v>
+        <v>0.63095238</v>
       </c>
       <c r="AD68" s="27" t="n">
-        <v>0.607142857142857</v>
+        <v>0.60714286</v>
       </c>
       <c r="AE68" s="27" t="n">
-        <v>0.595238095238095</v>
+        <v>0.5952381</v>
       </c>
       <c r="AF68" s="27" t="n">
-        <v>0.595238095238095</v>
+        <v>0.5952381</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20897,43 +20897,43 @@
         <v>1</v>
       </c>
       <c r="D69" s="27" t="n">
-        <v>0.983333333333333</v>
+        <v>0.98333333</v>
       </c>
       <c r="E69" s="27" t="n">
-        <v>0.983333333333333</v>
+        <v>0.98333333</v>
       </c>
       <c r="F69" s="27" t="n">
-        <v>0.966666666666667</v>
+        <v>0.96666667</v>
       </c>
       <c r="G69" s="27" t="n">
-        <v>0.966666666666667</v>
+        <v>0.96666667</v>
       </c>
       <c r="H69" s="27" t="n">
-        <v>0.966666666666667</v>
+        <v>0.96666667</v>
       </c>
       <c r="I69" s="27" t="n">
-        <v>0.966666666666667</v>
+        <v>0.96666667</v>
       </c>
       <c r="J69" s="27" t="n">
-        <v>0.933333333333333</v>
+        <v>0.93333333</v>
       </c>
       <c r="K69" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="L69" s="27" t="n">
-        <v>0.916666666666667</v>
+        <v>0.91666667</v>
       </c>
       <c r="M69" s="27" t="n">
         <v>0.9</v>
       </c>
       <c r="N69" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="O69" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="P69" s="27" t="n">
-        <v>0.883333333333333</v>
+        <v>0.88333333</v>
       </c>
       <c r="Q69" s="27" t="n">
         <v>0.85</v>
@@ -20951,16 +20951,16 @@
         <v>0.85</v>
       </c>
       <c r="V69" s="27" t="n">
-        <v>0.833333333333334</v>
+        <v>0.83333333</v>
       </c>
       <c r="W69" s="27" t="n">
-        <v>0.816666666666667</v>
+        <v>0.81666667</v>
       </c>
       <c r="X69" s="27" t="n">
         <v>0.8</v>
       </c>
       <c r="Y69" s="27" t="n">
-        <v>0.766666666666667</v>
+        <v>0.76666667</v>
       </c>
       <c r="Z69" s="27" t="n">
         <v>0.75</v>
@@ -20969,10 +20969,10 @@
         <v>0.75</v>
       </c>
       <c r="AB69" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
       <c r="AC69" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20992,67 +20992,67 @@
         <v>1</v>
       </c>
       <c r="F70" s="27" t="n">
-        <v>0.98780487804878</v>
+        <v>0.98780488</v>
       </c>
       <c r="G70" s="27" t="n">
-        <v>0.98780487804878</v>
+        <v>0.98780488</v>
       </c>
       <c r="H70" s="27" t="n">
-        <v>0.98780487804878</v>
+        <v>0.98780488</v>
       </c>
       <c r="I70" s="27" t="n">
-        <v>0.963414634146342</v>
+        <v>0.96341463</v>
       </c>
       <c r="J70" s="27" t="n">
-        <v>0.951219512195122</v>
+        <v>0.95121951</v>
       </c>
       <c r="K70" s="27" t="n">
-        <v>0.902439024390244</v>
+        <v>0.90243902</v>
       </c>
       <c r="L70" s="27" t="n">
-        <v>0.878048780487805</v>
+        <v>0.87804878</v>
       </c>
       <c r="M70" s="27" t="n">
-        <v>0.853658536585366</v>
+        <v>0.85365854</v>
       </c>
       <c r="N70" s="27" t="n">
-        <v>0.841463414634146</v>
+        <v>0.84146341</v>
       </c>
       <c r="O70" s="27" t="n">
-        <v>0.841463414634146</v>
+        <v>0.84146341</v>
       </c>
       <c r="P70" s="27" t="n">
-        <v>0.817073170731707</v>
+        <v>0.81707317</v>
       </c>
       <c r="Q70" s="27" t="n">
-        <v>0.804878048780488</v>
+        <v>0.80487805</v>
       </c>
       <c r="R70" s="27" t="n">
-        <v>0.780487804878049</v>
+        <v>0.7804878</v>
       </c>
       <c r="S70" s="27" t="n">
-        <v>0.768292682926829</v>
+        <v>0.76829268</v>
       </c>
       <c r="T70" s="27" t="n">
-        <v>0.768292682926829</v>
+        <v>0.76829268</v>
       </c>
       <c r="U70" s="27" t="n">
-        <v>0.75609756097561</v>
+        <v>0.75609756</v>
       </c>
       <c r="V70" s="27" t="n">
-        <v>0.75609756097561</v>
+        <v>0.75609756</v>
       </c>
       <c r="W70" s="27" t="n">
-        <v>0.75609756097561</v>
+        <v>0.75609756</v>
       </c>
       <c r="X70" s="27" t="n">
-        <v>0.74390243902439</v>
+        <v>0.74390244</v>
       </c>
       <c r="Y70" s="27" t="n">
-        <v>0.719512195121951</v>
+        <v>0.7195122</v>
       </c>
       <c r="Z70" s="27" t="n">
-        <v>0.695121951219512</v>
+        <v>0.69512195</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21066,52 +21066,52 @@
         <v>1</v>
       </c>
       <c r="D71" s="27" t="n">
-        <v>0.986666666666667</v>
+        <v>0.98666667</v>
       </c>
       <c r="E71" s="27" t="n">
-        <v>0.986666666666667</v>
+        <v>0.98666667</v>
       </c>
       <c r="F71" s="27" t="n">
-        <v>0.933333333333333</v>
+        <v>0.93333333</v>
       </c>
       <c r="G71" s="27" t="n">
-        <v>0.933333333333333</v>
+        <v>0.93333333</v>
       </c>
       <c r="H71" s="27" t="n">
-        <v>0.933333333333333</v>
+        <v>0.93333333</v>
       </c>
       <c r="I71" s="27" t="n">
-        <v>0.893333333333333</v>
+        <v>0.89333333</v>
       </c>
       <c r="J71" s="27" t="n">
-        <v>0.826666666666667</v>
+        <v>0.82666667</v>
       </c>
       <c r="K71" s="27" t="n">
         <v>0.8</v>
       </c>
       <c r="L71" s="27" t="n">
-        <v>0.786666666666667</v>
+        <v>0.78666667</v>
       </c>
       <c r="M71" s="27" t="n">
-        <v>0.786666666666667</v>
+        <v>0.78666667</v>
       </c>
       <c r="N71" s="27" t="n">
-        <v>0.786666666666667</v>
+        <v>0.78666667</v>
       </c>
       <c r="O71" s="27" t="n">
-        <v>0.773333333333333</v>
+        <v>0.77333333</v>
       </c>
       <c r="P71" s="27" t="n">
-        <v>0.773333333333333</v>
+        <v>0.77333333</v>
       </c>
       <c r="Q71" s="27" t="n">
-        <v>0.746666666666667</v>
+        <v>0.74666667</v>
       </c>
       <c r="R71" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
       <c r="S71" s="27" t="n">
-        <v>0.733333333333333</v>
+        <v>0.73333333</v>
       </c>
       <c r="T71" s="27" t="n">
         <v>0.72</v>
@@ -21123,7 +21123,7 @@
         <v>0.68</v>
       </c>
       <c r="W71" s="27" t="n">
-        <v>0.666666666666667</v>
+        <v>0.66666667</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21134,58 +21134,58 @@
         <v>1</v>
       </c>
       <c r="C72" s="27" t="n">
-        <v>0.98876404494382</v>
+        <v>0.98876404</v>
       </c>
       <c r="D72" s="27" t="n">
-        <v>0.97752808988764</v>
+        <v>0.97752809</v>
       </c>
       <c r="E72" s="27" t="n">
-        <v>0.966292134831461</v>
+        <v>0.96629213</v>
       </c>
       <c r="F72" s="27" t="n">
-        <v>0.932584269662921</v>
+        <v>0.93258427</v>
       </c>
       <c r="G72" s="27" t="n">
-        <v>0.887640449438202</v>
+        <v>0.88764045</v>
       </c>
       <c r="H72" s="27" t="n">
-        <v>0.876404494382023</v>
+        <v>0.87640449</v>
       </c>
       <c r="I72" s="27" t="n">
-        <v>0.842696629213483</v>
+        <v>0.84269663</v>
       </c>
       <c r="J72" s="27" t="n">
-        <v>0.808988764044944</v>
+        <v>0.80898876</v>
       </c>
       <c r="K72" s="27" t="n">
-        <v>0.764044943820225</v>
+        <v>0.76404494</v>
       </c>
       <c r="L72" s="27" t="n">
-        <v>0.752808988764045</v>
+        <v>0.75280899</v>
       </c>
       <c r="M72" s="27" t="n">
-        <v>0.752808988764045</v>
+        <v>0.75280899</v>
       </c>
       <c r="N72" s="27" t="n">
-        <v>0.730337078651685</v>
+        <v>0.73033708</v>
       </c>
       <c r="O72" s="27" t="n">
-        <v>0.707865168539326</v>
+        <v>0.70786517</v>
       </c>
       <c r="P72" s="27" t="n">
-        <v>0.674157303370787</v>
+        <v>0.6741573</v>
       </c>
       <c r="Q72" s="27" t="n">
-        <v>0.674157303370787</v>
+        <v>0.6741573</v>
       </c>
       <c r="R72" s="27" t="n">
-        <v>0.662921348314607</v>
+        <v>0.66292135</v>
       </c>
       <c r="S72" s="27" t="n">
-        <v>0.651685393258427</v>
+        <v>0.65168539</v>
       </c>
       <c r="T72" s="27" t="n">
-        <v>0.640449438202247</v>
+        <v>0.64044944</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21199,46 +21199,46 @@
         <v>1</v>
       </c>
       <c r="D73" s="27" t="n">
-        <v>0.984615384615385</v>
+        <v>0.98461538</v>
       </c>
       <c r="E73" s="27" t="n">
-        <v>0.984615384615385</v>
+        <v>0.98461538</v>
       </c>
       <c r="F73" s="27" t="n">
-        <v>0.984615384615385</v>
+        <v>0.98461538</v>
       </c>
       <c r="G73" s="27" t="n">
-        <v>0.984615384615385</v>
+        <v>0.98461538</v>
       </c>
       <c r="H73" s="27" t="n">
-        <v>0.953846153846154</v>
+        <v>0.95384615</v>
       </c>
       <c r="I73" s="27" t="n">
-        <v>0.938461538461538</v>
+        <v>0.93846154</v>
       </c>
       <c r="J73" s="27" t="n">
-        <v>0.861538461538462</v>
+        <v>0.86153846</v>
       </c>
       <c r="K73" s="27" t="n">
-        <v>0.830769230769231</v>
+        <v>0.83076923</v>
       </c>
       <c r="L73" s="27" t="n">
         <v>0.8</v>
       </c>
       <c r="M73" s="27" t="n">
-        <v>0.784615384615385</v>
+        <v>0.78461538</v>
       </c>
       <c r="N73" s="27" t="n">
-        <v>0.769230769230769</v>
+        <v>0.76923077</v>
       </c>
       <c r="O73" s="27" t="n">
-        <v>0.769230769230769</v>
+        <v>0.76923077</v>
       </c>
       <c r="P73" s="27" t="n">
-        <v>0.723076923076923</v>
+        <v>0.72307692</v>
       </c>
       <c r="Q73" s="27" t="n">
-        <v>0.707692307692308</v>
+        <v>0.70769231</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21249,40 +21249,40 @@
         <v>1</v>
       </c>
       <c r="C74" s="27" t="n">
-        <v>0.972972972972973</v>
+        <v>0.97297297</v>
       </c>
       <c r="D74" s="27" t="n">
-        <v>0.959459459459459</v>
+        <v>0.95945946</v>
       </c>
       <c r="E74" s="27" t="n">
-        <v>0.932432432432433</v>
+        <v>0.93243243</v>
       </c>
       <c r="F74" s="27" t="n">
-        <v>0.932432432432433</v>
+        <v>0.93243243</v>
       </c>
       <c r="G74" s="27" t="n">
-        <v>0.864864864864865</v>
+        <v>0.86486486</v>
       </c>
       <c r="H74" s="27" t="n">
-        <v>0.851351351351351</v>
+        <v>0.85135135</v>
       </c>
       <c r="I74" s="27" t="n">
-        <v>0.810810810810811</v>
+        <v>0.81081081</v>
       </c>
       <c r="J74" s="27" t="n">
-        <v>0.797297297297297</v>
+        <v>0.7972973</v>
       </c>
       <c r="K74" s="27" t="n">
-        <v>0.77027027027027</v>
+        <v>0.77027027</v>
       </c>
       <c r="L74" s="27" t="n">
-        <v>0.77027027027027</v>
+        <v>0.77027027</v>
       </c>
       <c r="M74" s="27" t="n">
-        <v>0.72972972972973</v>
+        <v>0.72972973</v>
       </c>
       <c r="N74" s="27" t="n">
-        <v>0.702702702702703</v>
+        <v>0.7027027</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21293,31 +21293,31 @@
         <v>1</v>
       </c>
       <c r="C75" s="27" t="n">
-        <v>0.978260869565217</v>
+        <v>0.97826087</v>
       </c>
       <c r="D75" s="27" t="n">
-        <v>0.956521739130435</v>
+        <v>0.95652174</v>
       </c>
       <c r="E75" s="27" t="n">
-        <v>0.945652173913044</v>
+        <v>0.94565217</v>
       </c>
       <c r="F75" s="27" t="n">
-        <v>0.902173913043478</v>
+        <v>0.90217391</v>
       </c>
       <c r="G75" s="27" t="n">
-        <v>0.891304347826087</v>
+        <v>0.89130435</v>
       </c>
       <c r="H75" s="27" t="n">
-        <v>0.869565217391304</v>
+        <v>0.86956522</v>
       </c>
       <c r="I75" s="27" t="n">
-        <v>0.858695652173913</v>
+        <v>0.85869565</v>
       </c>
       <c r="J75" s="27" t="n">
-        <v>0.847826086956522</v>
+        <v>0.84782609</v>
       </c>
       <c r="K75" s="27" t="n">
-        <v>0.836956521739131</v>
+        <v>0.83695652</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21331,19 +21331,19 @@
         <v>1</v>
       </c>
       <c r="D76" s="27" t="n">
-        <v>0.982142857142857</v>
+        <v>0.98214286</v>
       </c>
       <c r="E76" s="27" t="n">
-        <v>0.964285714285714</v>
+        <v>0.96428571</v>
       </c>
       <c r="F76" s="27" t="n">
-        <v>0.928571428571429</v>
+        <v>0.92857143</v>
       </c>
       <c r="G76" s="27" t="n">
-        <v>0.857142857142857</v>
+        <v>0.85714286</v>
       </c>
       <c r="H76" s="27" t="n">
-        <v>0.839285714285714</v>
+        <v>0.83928571</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21354,13 +21354,13 @@
         <v>1</v>
       </c>
       <c r="C77" s="27" t="n">
-        <v>0.989473684210526</v>
+        <v>0.98947368</v>
       </c>
       <c r="D77" s="27" t="n">
-        <v>0.968421052631579</v>
+        <v>0.96842105</v>
       </c>
       <c r="E77" s="27" t="n">
-        <v>0.968421052631579</v>
+        <v>0.96842105</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Step 6: Power BI build plan, measures and expected values
- dashboard/export_model_data.py: star-schema CSVs (FactRevenue,
  FactMRR, FactCost, DimCustomer, DimProduct, DimProductLine, DimDate)
  and expected_values.csv (624 rows: each year, year x product line,
  2025 x region group / region / size band)
- dashboard/measures.dax: 24 commented measures incl. NRR, GRR, logo
  churn, TOPN concentration, gross margin; slicer exceptions
- dashboard/README.md: relationships, why FactCost joins via a
  product-line dimension, page wireframes, slicers, build steps
- model_data CSVs are regenerated, not committed (D21)
- 4 new tests (88 in total)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LpN25NXzSEvizAa4wBvUc3
</commit_message>
<xml_diff>
--- a/databook/Northbridge_Databook.xlsx
+++ b/databook/Northbridge_Databook.xlsx
@@ -2900,11 +2900,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="68182179"/>
-        <c:axId val="30665427"/>
+        <c:axId val="82357641"/>
+        <c:axId val="89304075"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="68182179"/>
+        <c:axId val="82357641"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2970,7 +2970,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30665427"/>
+        <c:crossAx val="89304075"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2978,7 +2978,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30665427"/>
+        <c:axId val="89304075"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3044,7 +3044,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68182179"/>
+        <c:crossAx val="82357641"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3419,11 +3419,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="92032456"/>
-        <c:axId val="51481830"/>
+        <c:axId val="57525708"/>
+        <c:axId val="7638195"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="92032456"/>
+        <c:axId val="57525708"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3489,7 +3489,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51481830"/>
+        <c:crossAx val="7638195"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3497,7 +3497,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="51481830"/>
+        <c:axId val="7638195"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3563,7 +3563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92032456"/>
+        <c:crossAx val="57525708"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4051,11 +4051,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="80391956"/>
-        <c:axId val="61916199"/>
+        <c:axId val="14273169"/>
+        <c:axId val="14209071"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="80391956"/>
+        <c:axId val="14273169"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4121,7 +4121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61916199"/>
+        <c:crossAx val="14209071"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4129,7 +4129,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61916199"/>
+        <c:axId val="14209071"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4195,7 +4195,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80391956"/>
+        <c:crossAx val="14273169"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4656,11 +4656,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="11610500"/>
-        <c:axId val="97597414"/>
+        <c:axId val="28408486"/>
+        <c:axId val="40564505"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="11610500"/>
+        <c:axId val="28408486"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4726,7 +4726,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97597414"/>
+        <c:crossAx val="40564505"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4734,7 +4734,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="97597414"/>
+        <c:axId val="40564505"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4800,7 +4800,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11610500"/>
+        <c:crossAx val="28408486"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5157,11 +5157,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="99355520"/>
-        <c:axId val="79132325"/>
+        <c:axId val="27894174"/>
+        <c:axId val="17659662"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="99355520"/>
+        <c:axId val="27894174"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5227,7 +5227,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79132325"/>
+        <c:crossAx val="17659662"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5235,7 +5235,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79132325"/>
+        <c:axId val="17659662"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.1"/>
@@ -5303,7 +5303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99355520"/>
+        <c:crossAx val="27894174"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5890,11 +5890,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="90034550"/>
-        <c:axId val="44332542"/>
+        <c:axId val="8459537"/>
+        <c:axId val="75778823"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="90034550"/>
+        <c:axId val="8459537"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5926,7 +5926,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44332542"/>
+        <c:crossAx val="75778823"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5934,7 +5934,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44332542"/>
+        <c:axId val="75778823"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="25000000"/>
@@ -6001,7 +6001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90034550"/>
+        <c:crossAx val="8459537"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6489,11 +6489,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="47346770"/>
-        <c:axId val="39380636"/>
+        <c:axId val="7732728"/>
+        <c:axId val="95818143"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="47346770"/>
+        <c:axId val="7732728"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6559,7 +6559,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39380636"/>
+        <c:crossAx val="95818143"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6567,7 +6567,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="39380636"/>
+        <c:axId val="95818143"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6633,7 +6633,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47346770"/>
+        <c:crossAx val="7732728"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6819,11 +6819,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="62505300"/>
-        <c:axId val="49705050"/>
+        <c:axId val="52407254"/>
+        <c:axId val="9838636"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="62505300"/>
+        <c:axId val="52407254"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6855,7 +6855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49705050"/>
+        <c:crossAx val="9838636"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6863,7 +6863,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="49705050"/>
+        <c:axId val="9838636"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6929,7 +6929,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62505300"/>
+        <c:crossAx val="52407254"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Step 7: findings memo generated from the pipeline, two pages
- memo/build_memo.py writes memo/findings_memo.md and .docx and exports
  the PDF with LibreOffice; fails the build if it runs over two pages
- scope, key findings with databook tab references, rated red flags,
  adjusted views of 2025 revenue, 14 questions for management, and an
  overall view (proceed with price and structure protections) with each
  protection linked to a red flag
- every £ and % in the memo and key_findings.md is tested against
  outputs/tables/; memo and readme stages added to run_all.py
- decisions D23-D25; 4 new tests (92 in total)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LpN25NXzSEvizAa4wBvUc3
</commit_message>
<xml_diff>
--- a/databook/Northbridge_Databook.xlsx
+++ b/databook/Northbridge_Databook.xlsx
@@ -2900,11 +2900,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="82357641"/>
-        <c:axId val="89304075"/>
+        <c:axId val="72493507"/>
+        <c:axId val="66294804"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="82357641"/>
+        <c:axId val="72493507"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2970,7 +2970,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89304075"/>
+        <c:crossAx val="66294804"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2978,7 +2978,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89304075"/>
+        <c:axId val="66294804"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3044,7 +3044,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82357641"/>
+        <c:crossAx val="72493507"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3419,11 +3419,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="57525708"/>
-        <c:axId val="7638195"/>
+        <c:axId val="55445369"/>
+        <c:axId val="58622581"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57525708"/>
+        <c:axId val="55445369"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3489,7 +3489,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7638195"/>
+        <c:crossAx val="58622581"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3497,7 +3497,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7638195"/>
+        <c:axId val="58622581"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3563,7 +3563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57525708"/>
+        <c:crossAx val="55445369"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4051,11 +4051,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="14273169"/>
-        <c:axId val="14209071"/>
+        <c:axId val="37151644"/>
+        <c:axId val="29759461"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="14273169"/>
+        <c:axId val="37151644"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4121,7 +4121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14209071"/>
+        <c:crossAx val="29759461"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4129,7 +4129,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14209071"/>
+        <c:axId val="29759461"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4195,7 +4195,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14273169"/>
+        <c:crossAx val="37151644"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4656,11 +4656,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="28408486"/>
-        <c:axId val="40564505"/>
+        <c:axId val="40806491"/>
+        <c:axId val="28115496"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="28408486"/>
+        <c:axId val="40806491"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4726,7 +4726,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40564505"/>
+        <c:crossAx val="28115496"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4734,7 +4734,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40564505"/>
+        <c:axId val="28115496"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4800,7 +4800,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28408486"/>
+        <c:crossAx val="40806491"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5157,11 +5157,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="27894174"/>
-        <c:axId val="17659662"/>
+        <c:axId val="37012547"/>
+        <c:axId val="86619264"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="27894174"/>
+        <c:axId val="37012547"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5227,7 +5227,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17659662"/>
+        <c:crossAx val="86619264"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5235,7 +5235,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17659662"/>
+        <c:axId val="86619264"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.1"/>
@@ -5303,7 +5303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27894174"/>
+        <c:crossAx val="37012547"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5890,11 +5890,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="8459537"/>
-        <c:axId val="75778823"/>
+        <c:axId val="63662921"/>
+        <c:axId val="57595087"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="8459537"/>
+        <c:axId val="63662921"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5926,7 +5926,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75778823"/>
+        <c:crossAx val="57595087"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5934,7 +5934,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75778823"/>
+        <c:axId val="57595087"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="25000000"/>
@@ -6001,7 +6001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8459537"/>
+        <c:crossAx val="63662921"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6489,11 +6489,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="7732728"/>
-        <c:axId val="95818143"/>
+        <c:axId val="76381963"/>
+        <c:axId val="86883649"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="7732728"/>
+        <c:axId val="76381963"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6559,7 +6559,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95818143"/>
+        <c:crossAx val="86883649"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6567,7 +6567,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95818143"/>
+        <c:axId val="86883649"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6633,7 +6633,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7732728"/>
+        <c:crossAx val="76381963"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6819,11 +6819,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="52407254"/>
-        <c:axId val="9838636"/>
+        <c:axId val="54395973"/>
+        <c:axId val="93129291"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="52407254"/>
+        <c:axId val="54395973"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6855,7 +6855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9838636"/>
+        <c:crossAx val="93129291"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6863,7 +6863,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9838636"/>
+        <c:axId val="93129291"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6929,7 +6929,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52407254"/>
+        <c:crossAx val="54395973"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Overnight run complete: morning summary, Step 8 summary, v1.0
- docs/overnight_report.md: morning summary at the top (status by
  step, headline findings, planted issues, recommendation, decisions,
  limitations, hand steps, repo state, reading list, interview
  questions) and the Step 8 summary
- interview prep answers extended to 60-75 seconds spoken
- fresh-clone check: run_all.py exit 0 in 65.3s, 106 tests passed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LpN25NXzSEvizAa4wBvUc3
</commit_message>
<xml_diff>
--- a/databook/Northbridge_Databook.xlsx
+++ b/databook/Northbridge_Databook.xlsx
@@ -2900,11 +2900,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="72493507"/>
-        <c:axId val="66294804"/>
+        <c:axId val="9289899"/>
+        <c:axId val="61983956"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="72493507"/>
+        <c:axId val="9289899"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2970,7 +2970,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66294804"/>
+        <c:crossAx val="61983956"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2978,7 +2978,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66294804"/>
+        <c:axId val="61983956"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3044,7 +3044,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72493507"/>
+        <c:crossAx val="9289899"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3419,11 +3419,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="55445369"/>
-        <c:axId val="58622581"/>
+        <c:axId val="32273007"/>
+        <c:axId val="23551209"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="55445369"/>
+        <c:axId val="32273007"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3489,7 +3489,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58622581"/>
+        <c:crossAx val="23551209"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3497,7 +3497,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58622581"/>
+        <c:axId val="23551209"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3563,7 +3563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55445369"/>
+        <c:crossAx val="32273007"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4051,11 +4051,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="37151644"/>
-        <c:axId val="29759461"/>
+        <c:axId val="33440144"/>
+        <c:axId val="1451052"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="37151644"/>
+        <c:axId val="33440144"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4121,7 +4121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29759461"/>
+        <c:crossAx val="1451052"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4129,7 +4129,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29759461"/>
+        <c:axId val="1451052"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4195,7 +4195,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37151644"/>
+        <c:crossAx val="33440144"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4656,11 +4656,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="40806491"/>
-        <c:axId val="28115496"/>
+        <c:axId val="78867227"/>
+        <c:axId val="91023099"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="40806491"/>
+        <c:axId val="78867227"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4726,7 +4726,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28115496"/>
+        <c:crossAx val="91023099"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4734,7 +4734,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="28115496"/>
+        <c:axId val="91023099"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4800,7 +4800,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40806491"/>
+        <c:crossAx val="78867227"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5157,11 +5157,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="37012547"/>
-        <c:axId val="86619264"/>
+        <c:axId val="54285644"/>
+        <c:axId val="76058473"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="37012547"/>
+        <c:axId val="54285644"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5227,7 +5227,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86619264"/>
+        <c:crossAx val="76058473"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5235,7 +5235,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86619264"/>
+        <c:axId val="76058473"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.1"/>
@@ -5303,7 +5303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37012547"/>
+        <c:crossAx val="54285644"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5890,11 +5890,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="63662921"/>
-        <c:axId val="57595087"/>
+        <c:axId val="85370252"/>
+        <c:axId val="57348582"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="63662921"/>
+        <c:axId val="85370252"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5926,7 +5926,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57595087"/>
+        <c:crossAx val="57348582"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5934,7 +5934,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="57595087"/>
+        <c:axId val="57348582"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="25000000"/>
@@ -6001,7 +6001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63662921"/>
+        <c:crossAx val="85370252"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6489,11 +6489,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="76381963"/>
-        <c:axId val="86883649"/>
+        <c:axId val="26828430"/>
+        <c:axId val="96897188"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="76381963"/>
+        <c:axId val="26828430"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6559,7 +6559,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86883649"/>
+        <c:crossAx val="96897188"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6567,7 +6567,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86883649"/>
+        <c:axId val="96897188"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6633,7 +6633,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76381963"/>
+        <c:crossAx val="26828430"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6819,11 +6819,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="54395973"/>
-        <c:axId val="93129291"/>
+        <c:axId val="97462336"/>
+        <c:axId val="21696103"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="54395973"/>
+        <c:axId val="97462336"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6855,7 +6855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93129291"/>
+        <c:crossAx val="21696103"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6863,7 +6863,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93129291"/>
+        <c:axId val="21696103"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6929,7 +6929,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54395973"/>
+        <c:crossAx val="97462336"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Job 2 (WIP): deterministic reruns for notebooks, xlsx, docx and PDF
- report_config.json: document_date (the v1.0 release date) drives every
  file date.
- tools/normalise_ooxml.py, normalise_pdf.py, normalise_notebook.py fix
  the save-time stamps, random chart axis ids, zip layout, PDF /ID and
  /DocChecksum, and notebook timing metadata.
- run_all.py: PYTHONHASHSEED=0 for child processes, notebooks run without
  timing, --check-determinism flag.
- Explicit ORDER BY on exported and displayed queries; sorted() where a
  set fed a float sum; step 2 and 3 tables exported through save_table.
- outputs/tables and outputs/charts are byte-identical to v1.0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LpN25NXzSEvizAa4wBvUc3
</commit_message>
<xml_diff>
--- a/databook/Northbridge_Databook.xlsx
+++ b/databook/Northbridge_Databook.xlsx
@@ -2900,11 +2900,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="9289899"/>
-        <c:axId val="61983956"/>
+        <c:axId val="100001"/>
+        <c:axId val="100002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="9289899"/>
+        <c:axId val="100001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2970,7 +2970,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61983956"/>
+        <c:crossAx val="100002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2978,7 +2978,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61983956"/>
+        <c:axId val="100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3044,7 +3044,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9289899"/>
+        <c:crossAx val="100001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3419,11 +3419,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="32273007"/>
-        <c:axId val="23551209"/>
+        <c:axId val="100001"/>
+        <c:axId val="100002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="32273007"/>
+        <c:axId val="100001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3489,7 +3489,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23551209"/>
+        <c:crossAx val="100002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3497,7 +3497,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23551209"/>
+        <c:axId val="100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3563,7 +3563,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32273007"/>
+        <c:crossAx val="100001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4051,11 +4051,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="33440144"/>
-        <c:axId val="1451052"/>
+        <c:axId val="100001"/>
+        <c:axId val="100002"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="33440144"/>
+        <c:axId val="100001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4121,7 +4121,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1451052"/>
+        <c:crossAx val="100002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4129,7 +4129,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1451052"/>
+        <c:axId val="100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4195,7 +4195,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33440144"/>
+        <c:crossAx val="100001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4656,11 +4656,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="78867227"/>
-        <c:axId val="91023099"/>
+        <c:axId val="100001"/>
+        <c:axId val="100002"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="78867227"/>
+        <c:axId val="100001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4726,7 +4726,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91023099"/>
+        <c:crossAx val="100002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4734,7 +4734,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="91023099"/>
+        <c:axId val="100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4800,7 +4800,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78867227"/>
+        <c:crossAx val="100001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5157,11 +5157,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="54285644"/>
-        <c:axId val="76058473"/>
+        <c:axId val="100001"/>
+        <c:axId val="100002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="54285644"/>
+        <c:axId val="100001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5227,7 +5227,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76058473"/>
+        <c:crossAx val="100002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5235,7 +5235,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="76058473"/>
+        <c:axId val="100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1.1"/>
@@ -5303,7 +5303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54285644"/>
+        <c:crossAx val="100001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5890,11 +5890,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="85370252"/>
-        <c:axId val="57348582"/>
+        <c:axId val="100001"/>
+        <c:axId val="100002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="85370252"/>
+        <c:axId val="100001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5926,7 +5926,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57348582"/>
+        <c:crossAx val="100002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5934,7 +5934,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="57348582"/>
+        <c:axId val="100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="25000000"/>
@@ -6001,7 +6001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85370252"/>
+        <c:crossAx val="100001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6489,11 +6489,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="26828430"/>
-        <c:axId val="96897188"/>
+        <c:axId val="100001"/>
+        <c:axId val="100002"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="26828430"/>
+        <c:axId val="100001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6559,7 +6559,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96897188"/>
+        <c:crossAx val="100002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6567,7 +6567,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="96897188"/>
+        <c:axId val="100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6633,7 +6633,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26828430"/>
+        <c:crossAx val="100001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6819,11 +6819,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="97462336"/>
-        <c:axId val="21696103"/>
+        <c:axId val="100001"/>
+        <c:axId val="100002"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97462336"/>
+        <c:axId val="100001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6855,7 +6855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21696103"/>
+        <c:crossAx val="100002"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6863,7 +6863,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21696103"/>
+        <c:axId val="100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6929,7 +6929,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97462336"/>
+        <c:crossAx val="100001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Job 1 retry (D12): sourced SaaS retention benchmarks
Replace the indicative 4d ranges with figures read from SaaS Capital (2025,
2023 as context), High Alpha (2025), Benchmarkit (2025) and ChartMogul (2023,
context). The figures are a checked-in input, data/reference/benchmarks_source.csv,
which the 04d notebook validates and copies to outputs/tables/benchmarks.csv,
alongside a comparison table, a chart and docs/benchmarks.md.

Databook 4d, key finding F03, the memo (with a source footnote) and the
interview prep now quote the sourced figures. No rating or recommendation
changed. Decisions D12 and D28 resolved; new D35 to D39. Tests tie every
quoted benchmark figure to benchmarks.csv.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JYe5m76Q5dzWnkxrjnkzNA
</commit_message>
<xml_diff>
--- a/databook/Northbridge_Databook.xlsx
+++ b/databook/Northbridge_Databook.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="703">
   <si>
     <t xml:space="preserve">Project Northbridge</t>
   </si>
@@ -103,7 +103,7 @@
     <t xml:space="preserve">4d NRR GRR</t>
   </si>
   <si>
-    <t xml:space="preserve">NRR and GRR by year with sensitivities (excluding top 5, excluding price) and indicative benchmarks</t>
+    <t xml:space="preserve">NRR and GRR by year with sensitivities (excluding top 5, excluding price) and sourced SMB benchmarks</t>
   </si>
   <si>
     <t xml:space="preserve">4e ARR bridge</t>
@@ -355,7 +355,7 @@
     <t xml:space="preserve">- Margin by customer size depends on the cost allocation basis; the data room has no cost-to-serve driver.</t>
   </si>
   <si>
-    <t xml:space="preserve">- SaaS benchmark ranges on the 4d tab are indicative and not sourced.</t>
+    <t xml:space="preserve">- SaaS benchmarks on the 4d tab are survey medians whose definitions differ from ours in places (docs/benchmarks.md).</t>
   </si>
   <si>
     <t xml:space="preserve">- Customer lifecycle before 2022 relies on subscription dates; invoices before 2022 are not in the data room.</t>
@@ -1040,7 +1040,7 @@
     <t xml:space="preserve">Units: £'000 for MRR; % for NRR and GRR</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: outputs/tables/4d_nrr_grr.csv (notebooks/04d_nrr_grr.ipynb)</t>
+    <t xml:space="preserve">Source: outputs/tables/4d_nrr_grr.csv, benchmarks.csv, 4d_benchmark_comparison.csv (notebooks/04d_nrr_grr.ipynb)</t>
   </si>
   <si>
     <t xml:space="preserve">NRR and GRR (December to December MRR)</t>
@@ -1095,43 +1095,103 @@
   </si>
   <si>
     <t xml:space="preserve">DRAFT commentary for review (drafted from outputs/key_findings.md):
-F03 (High): Retention is weakening. NRR was 95.8%, 98.7% and 95.4% for 2023 to 2025; excluding the price increase it was 95.8%, 94.0% and 89.2%. GRR fell from 94.5% to 88.8%. Logo churn rose from 90 customers (8.9%) in 2023 to 171 (12.7%) in 2025. NRR and GRR are available for 2023 to 2025 only.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What good looks like for SMB-focused B2B SaaS (indicative, not sourced)</t>
+F03 (High): Retention is weakening. NRR was 95.8%, 98.7% and 95.4% for 2023 to 2025; excluding the price increase it was 95.8%, 94.0% and 89.2%. GRR fell from 94.5% to 88.8%. Logo churn rose from 90 customers (8.9%) in 2023 to 171 (12.7%) in 2025. NRR and GRR are available for 2023 to 2025 only. Against sourced benchmarks, 2025 NRR and GRR are below the SaaS Capital medians for SMB software, whose definitions match ours (98% to 103% NRR, 90% to 91% GRR), and NRR before the price increase is below every SMB median in the three 2025 benchmark surveys (94% to 107%; GRR medians 83% to 92%); see docs/benchmarks.md.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What good looks like: sourced SMB benchmarks (medians for ACV bands under US$50k; see docs/benchmarks.md)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Publisher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SC25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SaaS Capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV under $12k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV $12k to $25k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV $25k to $50k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HA25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High Alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV under $1k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV $1k to $5k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV $5k to $10k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV $10k to $15k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV $15k to $25k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BM25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benchmarkit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB: ACV $10k to $25k</t>
   </si>
   <si>
     <t xml:space="preserve">Measure</t>
   </si>
   <si>
-    <t xml:space="preserve">Weaker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">below 80%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">about 80% to 90%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">above 90%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">indicative, not sourced</t>
-  </si>
-  <si>
-    <t xml:space="preserve">below 90%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">about 90% to 105%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">above 105%</t>
+    <t xml:space="preserve">SMB median, low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMB median, high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SaaS Capital SMB median, low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SaaS Capital SMB median, high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northbridge 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per 4d notebook: low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per 4d notebook: high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRR before price increase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sources: SaaS Capital, 2025 B2B SaaS Retention Benchmarks (Research Brief 32) (2025), https://www.saas-capital.com/wp-content/uploads/2025/09/RB32WS1-2025-B2B-SaaS-Retention-Benchmarks.pdf, accessed 2026-09-26; High Alpha, 2025 SaaS Benchmarks Report (2025), https://2994607.fs1.hubspotusercontent-na1.net/hubfs/2994607/2025%20SaaS%20Benchmarks%20Report.pdf, accessed 2026-09-26; Benchmarkit, 2025 B2B SaaS Performance Metrics Benchmarks (2025), https://www.benchmarkit.ai/_files/ugd/2a084b_1b2e8054260b44cba36242807d1c3eea.pdf, accessed 2026-09-26. Only SaaS Capital uses our definitions (December-to-December MRR, price increases in NRR, GRR capped at opening MRR); the others do not state how price increases are treated. Bands are in US dollars; Northbridge's average ACV is in pounds. Medians place Northbridge in a distribution of private SaaS companies, largely US-based where stated; they are not a pass mark.</t>
   </si>
   <si>
     <t xml:space="preserve">4e. ARR bridge and revenue bridge</t>
@@ -1357,9 +1417,6 @@
     <t xml:space="preserve">Segments (flag: risk if logo churn is 5 points above the company rate or NRR 5 points below; small if fewer than 30 customers)</t>
   </si>
   <si>
-    <t xml:space="preserve">Segment</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dimension</t>
   </si>
   <si>
@@ -1965,6 +2022,15 @@
   </si>
   <si>
     <t xml:space="preserve">D20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4d NRR: SMB benchmark range recomputed from benchmarks.csv equals the 4d notebook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4d NRR before price increase: SMB benchmark range recomputed from benchmarks.csv equals the 4d notebook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4d GRR: SMB benchmark range recomputed from benchmarks.csv equals the 4d notebook</t>
   </si>
   <si>
     <t xml:space="preserve">4e ARR bridge 2023: opening plus components equals closing ARR from the cube</t>
@@ -2296,7 +2362,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2407,6 +2473,14 @@
     </xf>
     <xf numFmtId="174" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -7496,7 +7570,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>395</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7506,12 +7580,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>396</v>
+        <v>416</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>397</v>
+        <v>417</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7622,7 +7696,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>398</v>
+        <v>418</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7733,7 +7807,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>399</v>
+        <v>419</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7795,7 +7869,7 @@
         <v>3556345.12</v>
       </c>
       <c r="K24" s="22" t="s">
-        <v>400</v>
+        <v>420</v>
       </c>
       <c r="L24" s="22"/>
       <c r="M24" s="22"/>
@@ -7879,7 +7953,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>401</v>
+        <v>421</v>
       </c>
       <c r="K28" s="22"/>
       <c r="L28" s="22"/>
@@ -8050,7 +8124,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>402</v>
+        <v>422</v>
       </c>
       <c r="K35" s="22"/>
       <c r="L35" s="22"/>
@@ -8183,12 +8257,12 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="8" t="s">
-        <v>403</v>
+        <v>423</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>404</v>
+        <v>424</v>
       </c>
       <c r="B42" s="14" t="n">
         <f aca="false">B11-B19</f>
@@ -8209,28 +8283,28 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="B43" s="28" t="n">
+        <v>425</v>
+      </c>
+      <c r="B43" s="30" t="n">
         <f aca="false">B42/B11</f>
         <v>0.774474421886464</v>
       </c>
-      <c r="C43" s="28" t="n">
+      <c r="C43" s="30" t="n">
         <f aca="false">C42/C11</f>
         <v>0.773957755512257</v>
       </c>
-      <c r="D43" s="28" t="n">
+      <c r="D43" s="30" t="n">
         <f aca="false">D42/D11</f>
         <v>0.777876065021655</v>
       </c>
-      <c r="E43" s="28" t="n">
+      <c r="E43" s="30" t="n">
         <f aca="false">E42/E11</f>
         <v>0.737563955384109</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>406</v>
+        <v>426</v>
       </c>
       <c r="C44" s="24" t="n">
         <f aca="false">(C43-B43)*100</f>
@@ -8247,7 +8321,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>407</v>
+        <v>427</v>
       </c>
       <c r="C45" s="24" t="n">
         <f aca="false">SUMPRODUCT(C37:C40-B37:B40,B30:B33)*100</f>
@@ -8264,7 +8338,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>408</v>
+        <v>428</v>
       </c>
       <c r="C46" s="24" t="n">
         <f aca="false">SUMPRODUCT(C37:C40,C30:C33-B30:B33)*100</f>
@@ -8281,7 +8355,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>409</v>
+        <v>429</v>
       </c>
       <c r="C47" s="15" t="b">
         <f aca="false">ABS(C45+C46-C44)&lt;0.000001</f>
@@ -8298,7 +8372,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="s">
-        <v>410</v>
+        <v>430</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8320,7 +8394,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>411</v>
+        <v>431</v>
       </c>
       <c r="B51" s="11" t="n">
         <v>6367072.32</v>
@@ -8337,7 +8411,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>412</v>
+        <v>432</v>
       </c>
       <c r="B52" s="12" t="n">
         <f aca="false">B50-B51</f>
@@ -8358,7 +8432,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>413</v>
+        <v>433</v>
       </c>
       <c r="B53" s="12" t="n">
         <f aca="false">B42</f>
@@ -8400,7 +8474,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>414</v>
+        <v>434</v>
       </c>
       <c r="B55" s="18" t="n">
         <f aca="false">-SUMIFS(Reconciliation!$D$59:$D$62,Reconciliation!$A$59:$A$62,2022)</f>
@@ -8442,7 +8516,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="s">
-        <v>415</v>
+        <v>435</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8450,22 +8524,22 @@
         <v>114</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>416</v>
+        <v>436</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>417</v>
+        <v>437</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>418</v>
+        <v>438</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>419</v>
+        <v>439</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>420</v>
+        <v>440</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>421</v>
+        <v>441</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8578,32 +8652,32 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="8" t="s">
-        <v>422</v>
+        <v>442</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
-        <v>423</v>
+        <v>443</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>416</v>
+        <v>436</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>417</v>
+        <v>437</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>418</v>
+        <v>438</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>419</v>
+        <v>439</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>424</v>
+        <v>444</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="9" t="s">
-        <v>425</v>
+        <v>445</v>
       </c>
       <c r="B68" s="11" t="n">
         <v>4740760.6</v>
@@ -8626,7 +8700,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="9" t="s">
-        <v>426</v>
+        <v>446</v>
       </c>
       <c r="B69" s="11" t="n">
         <v>10781514.19</v>
@@ -8649,7 +8723,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="9" t="s">
-        <v>427</v>
+        <v>447</v>
       </c>
       <c r="B70" s="11" t="n">
         <v>11356310.18</v>
@@ -8672,7 +8746,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="9" t="s">
-        <v>428</v>
+        <v>448</v>
       </c>
       <c r="B71" s="11" t="n">
         <v>14005348.66</v>
@@ -8716,35 +8790,35 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="8" t="s">
-        <v>429</v>
+        <v>449</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="s">
-        <v>423</v>
+        <v>443</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>171</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>430</v>
+        <v>450</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>431</v>
+        <v>451</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>432</v>
+        <v>452</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>433</v>
+        <v>453</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>434</v>
+        <v>454</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="9" t="s">
-        <v>425</v>
+        <v>445</v>
       </c>
       <c r="B76" s="11" t="n">
         <v>5678883.83</v>
@@ -8769,7 +8843,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="9" t="s">
-        <v>426</v>
+        <v>446</v>
       </c>
       <c r="B77" s="11" t="n">
         <v>12761233.07</v>
@@ -8794,7 +8868,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="9" t="s">
-        <v>427</v>
+        <v>447</v>
       </c>
       <c r="B78" s="11" t="n">
         <v>12785193.46</v>
@@ -8819,7 +8893,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="9" t="s">
-        <v>428</v>
+        <v>448</v>
       </c>
       <c r="B79" s="11" t="n">
         <v>14531108.99</v>
@@ -8893,7 +8967,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>435</v>
+        <v>455</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8903,47 +8977,47 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>436</v>
+        <v>456</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>437</v>
+        <v>457</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>438</v>
+        <v>357</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>439</v>
+        <v>458</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>440</v>
+        <v>459</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>441</v>
+        <v>460</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>336</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>442</v>
+        <v>461</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>443</v>
+        <v>462</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>444</v>
+        <v>463</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>445</v>
+        <v>464</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>446</v>
+        <v>465</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>447</v>
+        <v>466</v>
       </c>
       <c r="L6" s="4" t="s">
         <v>339</v>
@@ -8952,15 +9026,15 @@
         <v>340</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>448</v>
+        <v>467</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>449</v>
+        <v>468</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>146</v>
@@ -9006,10 +9080,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>451</v>
+        <v>470</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>116</v>
@@ -9055,10 +9129,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>452</v>
+        <v>471</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>109</v>
@@ -9104,10 +9178,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>453</v>
+        <v>472</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>123</v>
@@ -9153,10 +9227,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>454</v>
+        <v>473</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>122</v>
@@ -9202,10 +9276,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>455</v>
+        <v>474</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>122</v>
@@ -9251,10 +9325,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>456</v>
+        <v>475</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>132</v>
@@ -9300,10 +9374,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>457</v>
+        <v>476</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>125</v>
@@ -9349,10 +9423,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>458</v>
+        <v>477</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C15" s="10" t="n">
         <v>135</v>
@@ -9398,10 +9472,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>459</v>
+        <v>478</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>132</v>
@@ -9447,10 +9521,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>460</v>
+        <v>479</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="C17" s="10" t="n">
         <v>81</v>
@@ -9496,10 +9570,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>461</v>
+        <v>480</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>462</v>
+        <v>481</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>95</v>
@@ -9545,10 +9619,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>463</v>
+        <v>482</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>462</v>
+        <v>481</v>
       </c>
       <c r="C19" s="10" t="n">
         <v>1248</v>
@@ -9594,10 +9668,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>464</v>
+        <v>483</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>465</v>
+        <v>484</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>384</v>
@@ -9643,10 +9717,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>466</v>
+        <v>485</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>465</v>
+        <v>484</v>
       </c>
       <c r="C21" s="10" t="n">
         <v>351</v>
@@ -9692,10 +9766,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>467</v>
+        <v>486</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>465</v>
+        <v>484</v>
       </c>
       <c r="C22" s="10" t="n">
         <v>221</v>
@@ -9741,10 +9815,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>468</v>
+        <v>487</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>465</v>
+        <v>484</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>223</v>
@@ -9790,10 +9864,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>469</v>
+        <v>488</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>465</v>
+        <v>484</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>164</v>
@@ -9837,7 +9911,7 @@
         <v>none</v>
       </c>
       <c r="P24" s="22" t="s">
-        <v>470</v>
+        <v>489</v>
       </c>
       <c r="Q24" s="22"/>
       <c r="R24" s="22"/>
@@ -9850,10 +9924,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>428</v>
+        <v>448</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>471</v>
+        <v>490</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>117</v>
@@ -9908,10 +9982,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>427</v>
+        <v>447</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>471</v>
+        <v>490</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>330</v>
@@ -9966,10 +10040,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>425</v>
+        <v>445</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>471</v>
+        <v>490</v>
       </c>
       <c r="C27" s="10" t="n">
         <v>353</v>
@@ -10024,10 +10098,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="s">
-        <v>426</v>
+        <v>446</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>471</v>
+        <v>490</v>
       </c>
       <c r="C28" s="10" t="n">
         <v>543</v>
@@ -10093,7 +10167,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>472</v>
+        <v>491</v>
       </c>
       <c r="C30" s="20" t="n">
         <f aca="false">SUMIFS(C$7:C$28,$B$7:$B$28,"industry")</f>
@@ -10123,19 +10197,19 @@
         <f aca="false">SUMIFS(I$7:I$28,$B$7:$B$28,"industry")</f>
         <v>45756419.35</v>
       </c>
-      <c r="J30" s="28" t="n">
+      <c r="J30" s="30" t="n">
         <f aca="false">I30/H30-1</f>
         <v>0.228066882807052</v>
       </c>
-      <c r="K30" s="28" t="n">
+      <c r="K30" s="30" t="n">
         <f aca="false">D30/C30</f>
         <v>0.127326880119136</v>
       </c>
-      <c r="L30" s="28" t="n">
+      <c r="L30" s="30" t="n">
         <f aca="false">F30/E30</f>
         <v>0.954434773207137</v>
       </c>
-      <c r="M30" s="28" t="n">
+      <c r="M30" s="30" t="n">
         <f aca="false">G30/E30</f>
         <v>0.887690505113145</v>
       </c>
@@ -10151,7 +10225,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>473</v>
+        <v>492</v>
       </c>
       <c r="C31" s="15" t="b">
         <f aca="false">AND(SUMIFS(C$7:C$28,$B$7:$B$28,"region_group")=C30,ABS(SUMIFS(I$7:I$28,$B$7:$B$28,"region_group")-I30)&lt;0.01)</f>
@@ -10169,7 +10243,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>474</v>
+        <v>493</v>
       </c>
       <c r="C32" s="15" t="b">
         <f aca="false">AND(SUMIFS(C$7:C$28,$B$7:$B$28,"acquisition_channel")=C30,ABS(SUMIFS(I$7:I$28,$B$7:$B$28,"acquisition_channel")-I30)&lt;0.01)</f>
@@ -10187,7 +10261,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>475</v>
+        <v>494</v>
       </c>
       <c r="C33" s="15" t="b">
         <f aca="false">AND(SUMIFS(C$7:C$28,$B$7:$B$28,"company_size")=C30,ABS(SUMIFS(I$7:I$28,$B$7:$B$28,"company_size")-I30)&lt;0.01)</f>
@@ -10205,7 +10279,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>476</v>
+        <v>495</v>
       </c>
       <c r="C34" s="15" t="b">
         <f aca="false">ABS(I30-'4a Revenue quality'!F10)&lt;0.01</f>
@@ -10264,523 +10338,523 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>477</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>478</v>
+        <v>497</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>479</v>
+        <v>498</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>480</v>
+        <v>499</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>481</v>
+        <v>500</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>482</v>
+        <v>501</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>483</v>
+        <v>502</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>484</v>
+        <v>503</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>485</v>
+        <v>504</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="29" t="s">
-        <v>486</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C6" s="29" t="s">
+      <c r="A6" s="31" t="s">
+        <v>505</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C6" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="D6" s="29" t="s">
-        <v>488</v>
-      </c>
-      <c r="E6" s="29" t="s">
-        <v>489</v>
-      </c>
-      <c r="F6" s="29" t="s">
-        <v>490</v>
-      </c>
-      <c r="G6" s="29" t="s">
-        <v>491</v>
+      <c r="D6" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>508</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>509</v>
+      </c>
+      <c r="G6" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
-        <v>492</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C7" s="29" t="s">
+      <c r="A7" s="31" t="s">
+        <v>511</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C7" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="29" t="s">
-        <v>493</v>
-      </c>
-      <c r="E7" s="29" t="s">
-        <v>494</v>
-      </c>
-      <c r="F7" s="29" t="s">
-        <v>495</v>
-      </c>
-      <c r="G7" s="29" t="s">
-        <v>491</v>
+      <c r="D7" s="31" t="s">
+        <v>512</v>
+      </c>
+      <c r="E7" s="31" t="s">
+        <v>513</v>
+      </c>
+      <c r="F7" s="31" t="s">
+        <v>514</v>
+      </c>
+      <c r="G7" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="29" t="s">
-        <v>496</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C8" s="29" t="s">
+      <c r="A8" s="31" t="s">
+        <v>515</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C8" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D8" s="29" t="s">
-        <v>493</v>
-      </c>
-      <c r="E8" s="29" t="s">
-        <v>497</v>
-      </c>
-      <c r="F8" s="29" t="s">
-        <v>498</v>
-      </c>
-      <c r="G8" s="29" t="s">
-        <v>491</v>
+      <c r="D8" s="31" t="s">
+        <v>512</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>516</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>517</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="s">
-        <v>499</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C9" s="29" t="s">
+      <c r="A9" s="31" t="s">
+        <v>518</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C9" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D9" s="29" t="s">
-        <v>493</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>500</v>
-      </c>
-      <c r="F9" s="29" t="s">
-        <v>501</v>
-      </c>
-      <c r="G9" s="29" t="s">
-        <v>491</v>
+      <c r="D9" s="31" t="s">
+        <v>512</v>
+      </c>
+      <c r="E9" s="31" t="s">
+        <v>519</v>
+      </c>
+      <c r="F9" s="31" t="s">
+        <v>520</v>
+      </c>
+      <c r="G9" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="s">
-        <v>502</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C10" s="29" t="s">
+      <c r="A10" s="31" t="s">
+        <v>521</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C10" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="D10" s="29" t="s">
-        <v>493</v>
-      </c>
-      <c r="E10" s="29" t="s">
-        <v>503</v>
-      </c>
-      <c r="F10" s="29" t="s">
-        <v>504</v>
-      </c>
-      <c r="G10" s="29" t="s">
-        <v>491</v>
+      <c r="D10" s="31" t="s">
+        <v>512</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>522</v>
+      </c>
+      <c r="F10" s="31" t="s">
+        <v>523</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="29" t="s">
-        <v>505</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C11" s="29" t="s">
+      <c r="A11" s="31" t="s">
+        <v>524</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C11" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="29" t="s">
+      <c r="D11" s="31" t="s">
+        <v>525</v>
+      </c>
+      <c r="E11" s="31" t="s">
+        <v>526</v>
+      </c>
+      <c r="F11" s="31" t="s">
+        <v>527</v>
+      </c>
+      <c r="G11" s="31" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="31" t="s">
+        <v>528</v>
+      </c>
+      <c r="B12" s="31" t="s">
         <v>506</v>
       </c>
-      <c r="E11" s="29" t="s">
-        <v>507</v>
-      </c>
-      <c r="F11" s="29" t="s">
-        <v>508</v>
-      </c>
-      <c r="G11" s="29" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="29" t="s">
-        <v>509</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="D12" s="29" t="s">
+      <c r="D12" s="31" t="s">
+        <v>529</v>
+      </c>
+      <c r="E12" s="31" t="s">
+        <v>530</v>
+      </c>
+      <c r="F12" s="31" t="s">
+        <v>531</v>
+      </c>
+      <c r="G12" s="31" t="s">
         <v>510</v>
       </c>
-      <c r="E12" s="29" t="s">
-        <v>511</v>
-      </c>
-      <c r="F12" s="29" t="s">
-        <v>512</v>
-      </c>
-      <c r="G12" s="29" t="s">
-        <v>491</v>
-      </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="s">
-        <v>513</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C13" s="29" t="s">
+      <c r="A13" s="31" t="s">
+        <v>532</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C13" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="D13" s="29" t="s">
-        <v>514</v>
-      </c>
-      <c r="E13" s="29" t="s">
-        <v>515</v>
-      </c>
-      <c r="F13" s="29" t="s">
-        <v>516</v>
-      </c>
-      <c r="G13" s="29" t="s">
-        <v>491</v>
+      <c r="D13" s="31" t="s">
+        <v>533</v>
+      </c>
+      <c r="E13" s="31" t="s">
+        <v>534</v>
+      </c>
+      <c r="F13" s="31" t="s">
+        <v>535</v>
+      </c>
+      <c r="G13" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29" t="s">
-        <v>517</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C14" s="29" t="s">
+      <c r="A14" s="31" t="s">
+        <v>536</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C14" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="D14" s="29" t="s">
-        <v>518</v>
-      </c>
-      <c r="E14" s="29" t="s">
-        <v>519</v>
-      </c>
-      <c r="F14" s="29" t="s">
-        <v>520</v>
-      </c>
-      <c r="G14" s="29" t="s">
-        <v>491</v>
+      <c r="D14" s="31" t="s">
+        <v>537</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>538</v>
+      </c>
+      <c r="F14" s="31" t="s">
+        <v>539</v>
+      </c>
+      <c r="G14" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29" t="s">
-        <v>521</v>
-      </c>
-      <c r="B15" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C15" s="29" t="s">
+      <c r="A15" s="31" t="s">
+        <v>540</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>506</v>
+      </c>
+      <c r="C15" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="D15" s="29" t="s">
-        <v>522</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>523</v>
-      </c>
-      <c r="F15" s="29" t="s">
-        <v>524</v>
-      </c>
-      <c r="G15" s="29" t="s">
-        <v>491</v>
+      <c r="D15" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>542</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>543</v>
+      </c>
+      <c r="G15" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29" t="s">
-        <v>525</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>526</v>
-      </c>
-      <c r="C16" s="29" t="s">
+      <c r="A16" s="31" t="s">
+        <v>544</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>545</v>
+      </c>
+      <c r="C16" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="D16" s="29" t="s">
-        <v>514</v>
-      </c>
-      <c r="E16" s="29" t="s">
-        <v>527</v>
-      </c>
-      <c r="F16" s="29" t="s">
-        <v>528</v>
-      </c>
-      <c r="G16" s="29" t="s">
-        <v>491</v>
+      <c r="D16" s="31" t="s">
+        <v>533</v>
+      </c>
+      <c r="E16" s="31" t="s">
+        <v>546</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>547</v>
+      </c>
+      <c r="G16" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="31" t="s">
+        <v>548</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>545</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" s="31" t="s">
         <v>529</v>
       </c>
-      <c r="B17" s="29" t="s">
-        <v>526</v>
-      </c>
-      <c r="C17" s="29" t="s">
+      <c r="E17" s="31" t="s">
+        <v>549</v>
+      </c>
+      <c r="F17" s="31" t="s">
+        <v>550</v>
+      </c>
+      <c r="G17" s="31" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="31" t="s">
+        <v>551</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>545</v>
+      </c>
+      <c r="C18" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="D18" s="31" t="s">
+        <v>529</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>552</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>553</v>
+      </c>
+      <c r="G18" s="31" t="s">
         <v>510</v>
       </c>
-      <c r="E17" s="29" t="s">
-        <v>530</v>
-      </c>
-      <c r="F17" s="29" t="s">
-        <v>531</v>
-      </c>
-      <c r="G17" s="29" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29" t="s">
-        <v>532</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>526</v>
-      </c>
-      <c r="C18" s="29" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="31" t="s">
+        <v>554</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>545</v>
+      </c>
+      <c r="C19" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="29" t="s">
+      <c r="D19" s="31" t="s">
+        <v>529</v>
+      </c>
+      <c r="E19" s="31" t="s">
+        <v>555</v>
+      </c>
+      <c r="F19" s="31" t="s">
+        <v>556</v>
+      </c>
+      <c r="G19" s="31" t="s">
         <v>510</v>
       </c>
-      <c r="E18" s="29" t="s">
-        <v>533</v>
-      </c>
-      <c r="F18" s="29" t="s">
-        <v>534</v>
-      </c>
-      <c r="G18" s="29" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="29" t="s">
-        <v>535</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>526</v>
-      </c>
-      <c r="C19" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="D19" s="29" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="31" t="s">
+        <v>557</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>559</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>560</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>561</v>
+      </c>
+      <c r="G20" s="31" t="s">
         <v>510</v>
       </c>
-      <c r="E19" s="29" t="s">
-        <v>536</v>
-      </c>
-      <c r="F19" s="29" t="s">
-        <v>537</v>
-      </c>
-      <c r="G19" s="29" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="29" t="s">
-        <v>538</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>539</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>540</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>541</v>
-      </c>
-      <c r="F20" s="29" t="s">
-        <v>542</v>
-      </c>
-      <c r="G20" s="29" t="s">
-        <v>491</v>
-      </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29" t="s">
-        <v>543</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>539</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>544</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>545</v>
-      </c>
-      <c r="E21" s="29" t="s">
-        <v>546</v>
-      </c>
-      <c r="F21" s="29" t="s">
-        <v>547</v>
-      </c>
-      <c r="G21" s="29" t="s">
-        <v>491</v>
+      <c r="A21" s="31" t="s">
+        <v>562</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="C21" s="31" t="s">
+        <v>563</v>
+      </c>
+      <c r="D21" s="31" t="s">
+        <v>564</v>
+      </c>
+      <c r="E21" s="31" t="s">
+        <v>565</v>
+      </c>
+      <c r="F21" s="31" t="s">
+        <v>566</v>
+      </c>
+      <c r="G21" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="29" t="s">
-        <v>548</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>539</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>544</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>545</v>
-      </c>
-      <c r="E22" s="29" t="s">
-        <v>549</v>
-      </c>
-      <c r="F22" s="29" t="s">
-        <v>550</v>
-      </c>
-      <c r="G22" s="29" t="s">
-        <v>491</v>
+      <c r="A22" s="31" t="s">
+        <v>567</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>563</v>
+      </c>
+      <c r="D22" s="31" t="s">
+        <v>564</v>
+      </c>
+      <c r="E22" s="31" t="s">
+        <v>568</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>569</v>
+      </c>
+      <c r="G22" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="29" t="s">
-        <v>551</v>
-      </c>
-      <c r="B23" s="29" t="s">
-        <v>539</v>
-      </c>
-      <c r="C23" s="29" t="s">
-        <v>552</v>
-      </c>
-      <c r="D23" s="29" t="s">
+      <c r="A23" s="31" t="s">
+        <v>570</v>
+      </c>
+      <c r="B23" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>571</v>
+      </c>
+      <c r="D23" s="31" t="s">
         <v>253</v>
       </c>
-      <c r="E23" s="29" t="s">
-        <v>553</v>
-      </c>
-      <c r="F23" s="29" t="s">
-        <v>554</v>
-      </c>
-      <c r="G23" s="29" t="s">
-        <v>491</v>
+      <c r="E23" s="31" t="s">
+        <v>572</v>
+      </c>
+      <c r="F23" s="31" t="s">
+        <v>573</v>
+      </c>
+      <c r="G23" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="29" t="s">
-        <v>555</v>
-      </c>
-      <c r="B24" s="29" t="s">
-        <v>539</v>
-      </c>
-      <c r="C24" s="29" t="s">
-        <v>556</v>
-      </c>
-      <c r="D24" s="29" t="s">
+      <c r="A24" s="31" t="s">
+        <v>574</v>
+      </c>
+      <c r="B24" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="C24" s="31" t="s">
+        <v>575</v>
+      </c>
+      <c r="D24" s="31" t="s">
         <v>253</v>
       </c>
-      <c r="E24" s="29" t="s">
-        <v>557</v>
-      </c>
-      <c r="F24" s="29" t="s">
+      <c r="E24" s="31" t="s">
+        <v>576</v>
+      </c>
+      <c r="F24" s="31" t="s">
+        <v>577</v>
+      </c>
+      <c r="G24" s="31" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="31" t="s">
+        <v>578</v>
+      </c>
+      <c r="B25" s="31" t="s">
         <v>558</v>
       </c>
-      <c r="G24" s="29" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="29" t="s">
-        <v>559</v>
-      </c>
-      <c r="B25" s="29" t="s">
-        <v>539</v>
-      </c>
-      <c r="C25" s="29" t="s">
-        <v>560</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>561</v>
-      </c>
-      <c r="E25" s="29" t="s">
-        <v>562</v>
-      </c>
-      <c r="F25" s="29" t="s">
-        <v>563</v>
-      </c>
-      <c r="G25" s="29" t="s">
-        <v>491</v>
+      <c r="C25" s="31" t="s">
+        <v>579</v>
+      </c>
+      <c r="D25" s="31" t="s">
+        <v>580</v>
+      </c>
+      <c r="E25" s="31" t="s">
+        <v>581</v>
+      </c>
+      <c r="F25" s="31" t="s">
+        <v>582</v>
+      </c>
+      <c r="G25" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="29" t="s">
-        <v>564</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>539</v>
-      </c>
-      <c r="C26" s="29" t="s">
-        <v>560</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>565</v>
-      </c>
-      <c r="E26" s="29" t="s">
-        <v>566</v>
-      </c>
-      <c r="F26" s="29" t="s">
-        <v>567</v>
-      </c>
-      <c r="G26" s="29" t="s">
-        <v>491</v>
+      <c r="A26" s="31" t="s">
+        <v>583</v>
+      </c>
+      <c r="B26" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>579</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>584</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>585</v>
+      </c>
+      <c r="F26" s="31" t="s">
+        <v>586</v>
+      </c>
+      <c r="G26" s="31" t="s">
+        <v>510</v>
       </c>
     </row>
   </sheetData>
@@ -10799,7 +10873,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -10810,31 +10884,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>568</v>
+        <v>587</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>569</v>
+        <v>588</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>570</v>
+        <v>589</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>571</v>
-      </c>
-      <c r="C5" s="30" t="b">
-        <f aca="false">AND(E8:E60)</f>
+        <v>590</v>
+      </c>
+      <c r="C5" s="32" t="b">
+        <f aca="false">AND(E8:E63)</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>572</v>
+        <v>591</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>145</v>
@@ -10843,10 +10917,10 @@
         <v>10</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>573</v>
+        <v>592</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>574</v>
+        <v>593</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10854,15 +10928,15 @@
         <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>575</v>
+        <v>594</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>576</v>
-      </c>
-      <c r="E8" s="31" t="b">
+        <v>595</v>
+      </c>
+      <c r="E8" s="33" t="b">
         <f aca="false">Reconciliation!I55</f>
         <v>1</v>
       </c>
@@ -10872,15 +10946,15 @@
         <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>577</v>
+        <v>596</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>578</v>
-      </c>
-      <c r="E9" s="31" t="b">
+        <v>597</v>
+      </c>
+      <c r="E9" s="33" t="b">
         <f aca="false">Reconciliation!I59</f>
         <v>1</v>
       </c>
@@ -10890,15 +10964,15 @@
         <v>3</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>579</v>
+        <v>598</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>580</v>
-      </c>
-      <c r="E10" s="31" t="b">
+        <v>599</v>
+      </c>
+      <c r="E10" s="33" t="b">
         <f aca="false">Reconciliation!I60</f>
         <v>1</v>
       </c>
@@ -10908,15 +10982,15 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>581</v>
+        <v>600</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>582</v>
-      </c>
-      <c r="E11" s="31" t="b">
+        <v>601</v>
+      </c>
+      <c r="E11" s="33" t="b">
         <f aca="false">Reconciliation!I61</f>
         <v>1</v>
       </c>
@@ -10926,15 +11000,15 @@
         <v>5</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>583</v>
+        <v>602</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="E12" s="31" t="b">
+        <v>603</v>
+      </c>
+      <c r="E12" s="33" t="b">
         <f aca="false">Reconciliation!I62</f>
         <v>1</v>
       </c>
@@ -10944,15 +11018,15 @@
         <v>6</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>585</v>
+        <v>604</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>586</v>
-      </c>
-      <c r="E13" s="31" t="b">
+        <v>605</v>
+      </c>
+      <c r="E13" s="33" t="b">
         <f aca="false">Reconciliation!B74</f>
         <v>1</v>
       </c>
@@ -10962,15 +11036,15 @@
         <v>7</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>587</v>
+        <v>606</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>588</v>
-      </c>
-      <c r="E14" s="31" t="b">
+        <v>607</v>
+      </c>
+      <c r="E14" s="33" t="b">
         <f aca="false">Reconciliation!C74</f>
         <v>1</v>
       </c>
@@ -10980,15 +11054,15 @@
         <v>8</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>589</v>
+        <v>608</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>590</v>
-      </c>
-      <c r="E15" s="31" t="b">
+        <v>609</v>
+      </c>
+      <c r="E15" s="33" t="b">
         <f aca="false">Reconciliation!D74</f>
         <v>1</v>
       </c>
@@ -10998,15 +11072,15 @@
         <v>9</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>591</v>
+        <v>610</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>592</v>
-      </c>
-      <c r="E16" s="31" t="b">
+        <v>611</v>
+      </c>
+      <c r="E16" s="33" t="b">
         <f aca="false">Reconciliation!E74</f>
         <v>1</v>
       </c>
@@ -11016,15 +11090,15 @@
         <v>10</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>593</v>
+        <v>612</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>594</v>
-      </c>
-      <c r="E17" s="31" t="b">
+        <v>613</v>
+      </c>
+      <c r="E17" s="33" t="b">
         <f aca="false">Reconciliation!F95</f>
         <v>1</v>
       </c>
@@ -11034,15 +11108,15 @@
         <v>11</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>595</v>
+        <v>614</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>596</v>
-      </c>
-      <c r="E18" s="31" t="b">
+        <v>615</v>
+      </c>
+      <c r="E18" s="33" t="b">
         <f aca="false">'4a Revenue quality'!N7</f>
         <v>1</v>
       </c>
@@ -11052,15 +11126,15 @@
         <v>12</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>597</v>
+        <v>616</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>598</v>
-      </c>
-      <c r="E19" s="31" t="b">
+        <v>617</v>
+      </c>
+      <c r="E19" s="33" t="b">
         <f aca="false">'4a Revenue quality'!N8</f>
         <v>1</v>
       </c>
@@ -11070,15 +11144,15 @@
         <v>13</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>599</v>
+        <v>618</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>600</v>
-      </c>
-      <c r="E20" s="31" t="b">
+        <v>619</v>
+      </c>
+      <c r="E20" s="33" t="b">
         <f aca="false">'4a Revenue quality'!N9</f>
         <v>1</v>
       </c>
@@ -11088,15 +11162,15 @@
         <v>14</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>601</v>
+        <v>620</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>602</v>
-      </c>
-      <c r="E21" s="31" t="b">
+        <v>621</v>
+      </c>
+      <c r="E21" s="33" t="b">
         <f aca="false">'4a Revenue quality'!N10</f>
         <v>1</v>
       </c>
@@ -11106,15 +11180,15 @@
         <v>15</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>603</v>
+        <v>622</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="E22" s="31" t="b">
+        <v>623</v>
+      </c>
+      <c r="E22" s="33" t="b">
         <f aca="false">'4b Concentration'!J7</f>
         <v>1</v>
       </c>
@@ -11124,15 +11198,15 @@
         <v>16</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>605</v>
+        <v>624</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="E23" s="31" t="b">
+        <v>625</v>
+      </c>
+      <c r="E23" s="33" t="b">
         <f aca="false">'4b Concentration'!J8</f>
         <v>1</v>
       </c>
@@ -11142,15 +11216,15 @@
         <v>17</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>607</v>
+        <v>626</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>608</v>
-      </c>
-      <c r="E24" s="31" t="b">
+        <v>627</v>
+      </c>
+      <c r="E24" s="33" t="b">
         <f aca="false">'4b Concentration'!J9</f>
         <v>1</v>
       </c>
@@ -11160,15 +11234,15 @@
         <v>18</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>609</v>
+        <v>628</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="E25" s="31" t="b">
+        <v>629</v>
+      </c>
+      <c r="E25" s="33" t="b">
         <f aca="false">'4b Concentration'!J10</f>
         <v>1</v>
       </c>
@@ -11178,15 +11252,15 @@
         <v>19</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>611</v>
+        <v>630</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>612</v>
-      </c>
-      <c r="E26" s="31" t="b">
+        <v>631</v>
+      </c>
+      <c r="E26" s="33" t="b">
         <f aca="false">'4b Concentration'!J11</f>
         <v>1</v>
       </c>
@@ -11196,15 +11270,15 @@
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>613</v>
+        <v>632</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>614</v>
-      </c>
-      <c r="E27" s="31" t="b">
+        <v>633</v>
+      </c>
+      <c r="E27" s="33" t="b">
         <f aca="false">'4b Concentration'!J12</f>
         <v>1</v>
       </c>
@@ -11214,15 +11288,15 @@
         <v>21</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>615</v>
+        <v>634</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="E28" s="31" t="b">
+        <v>635</v>
+      </c>
+      <c r="E28" s="33" t="b">
         <f aca="false">'4b Concentration'!J13</f>
         <v>1</v>
       </c>
@@ -11232,15 +11306,15 @@
         <v>22</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>617</v>
+        <v>636</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>618</v>
-      </c>
-      <c r="E29" s="31" t="b">
+        <v>637</v>
+      </c>
+      <c r="E29" s="33" t="b">
         <f aca="false">'4b Concentration'!J14</f>
         <v>1</v>
       </c>
@@ -11250,15 +11324,15 @@
         <v>23</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>619</v>
+        <v>638</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="E30" s="31" t="b">
+        <v>639</v>
+      </c>
+      <c r="E30" s="33" t="b">
         <f aca="false">'4b Concentration'!J15</f>
         <v>1</v>
       </c>
@@ -11268,15 +11342,15 @@
         <v>24</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>621</v>
+        <v>640</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>622</v>
-      </c>
-      <c r="E31" s="31" t="b">
+        <v>641</v>
+      </c>
+      <c r="E31" s="33" t="b">
         <f aca="false">'4b Concentration'!J16</f>
         <v>1</v>
       </c>
@@ -11286,15 +11360,15 @@
         <v>25</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>623</v>
+        <v>642</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="E32" s="31" t="b">
+        <v>643</v>
+      </c>
+      <c r="E32" s="33" t="b">
         <f aca="false">'4b Concentration'!J17</f>
         <v>1</v>
       </c>
@@ -11304,15 +11378,15 @@
         <v>26</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>625</v>
+        <v>644</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>626</v>
-      </c>
-      <c r="E33" s="31" t="b">
+        <v>645</v>
+      </c>
+      <c r="E33" s="33" t="b">
         <f aca="false">'4b Concentration'!J18</f>
         <v>1</v>
       </c>
@@ -11322,15 +11396,15 @@
         <v>27</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>627</v>
+        <v>646</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>628</v>
-      </c>
-      <c r="E34" s="31" t="b">
+        <v>647</v>
+      </c>
+      <c r="E34" s="33" t="b">
         <f aca="false">'4b Concentration'!J19</f>
         <v>1</v>
       </c>
@@ -11340,15 +11414,15 @@
         <v>28</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>629</v>
+        <v>648</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>630</v>
-      </c>
-      <c r="E35" s="31" t="b">
+        <v>649</v>
+      </c>
+      <c r="E35" s="33" t="b">
         <f aca="false">'4b Concentration'!J20</f>
         <v>1</v>
       </c>
@@ -11358,15 +11432,15 @@
         <v>29</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>631</v>
+        <v>650</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>632</v>
-      </c>
-      <c r="E36" s="31" t="b">
+        <v>651</v>
+      </c>
+      <c r="E36" s="33" t="b">
         <f aca="false">'4b Concentration'!J21</f>
         <v>1</v>
       </c>
@@ -11376,15 +11450,15 @@
         <v>30</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>633</v>
+        <v>652</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="E37" s="31" t="b">
+        <v>653</v>
+      </c>
+      <c r="E37" s="33" t="b">
         <f aca="false">'4b Concentration'!J22</f>
         <v>1</v>
       </c>
@@ -11394,15 +11468,15 @@
         <v>31</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>635</v>
+        <v>654</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>636</v>
-      </c>
-      <c r="E38" s="31" t="b">
+        <v>655</v>
+      </c>
+      <c r="E38" s="33" t="b">
         <f aca="false">'4d NRR GRR'!B20</f>
         <v>1</v>
       </c>
@@ -11412,15 +11486,15 @@
         <v>32</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>637</v>
+        <v>656</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>638</v>
-      </c>
-      <c r="E39" s="31" t="b">
+        <v>657</v>
+      </c>
+      <c r="E39" s="33" t="b">
         <f aca="false">'4d NRR GRR'!C20</f>
         <v>1</v>
       </c>
@@ -11430,15 +11504,15 @@
         <v>33</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>639</v>
+        <v>658</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>640</v>
-      </c>
-      <c r="E40" s="31" t="b">
+        <v>659</v>
+      </c>
+      <c r="E40" s="33" t="b">
         <f aca="false">'4d NRR GRR'!D20</f>
         <v>1</v>
       </c>
@@ -11448,16 +11522,16 @@
         <v>34</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>641</v>
+        <v>660</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>642</v>
-      </c>
-      <c r="E41" s="31" t="b">
-        <f aca="false">'4e ARR bridge'!B17</f>
+        <v>599</v>
+      </c>
+      <c r="E41" s="33" t="b">
+        <f aca="false">'4d NRR GRR'!I60</f>
         <v>1</v>
       </c>
     </row>
@@ -11466,16 +11540,16 @@
         <v>35</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>643</v>
+        <v>661</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>644</v>
-      </c>
-      <c r="E42" s="31" t="b">
-        <f aca="false">'4e ARR bridge'!C17</f>
+        <v>601</v>
+      </c>
+      <c r="E42" s="33" t="b">
+        <f aca="false">'4d NRR GRR'!I61</f>
         <v>1</v>
       </c>
     </row>
@@ -11484,16 +11558,16 @@
         <v>36</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>645</v>
+        <v>662</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>646</v>
-      </c>
-      <c r="E43" s="31" t="b">
-        <f aca="false">'4e ARR bridge'!D17</f>
+        <v>603</v>
+      </c>
+      <c r="E43" s="33" t="b">
+        <f aca="false">'4d NRR GRR'!I62</f>
         <v>1</v>
       </c>
     </row>
@@ -11502,16 +11576,16 @@
         <v>37</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>647</v>
+        <v>663</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>648</v>
-      </c>
-      <c r="E44" s="31" t="b">
-        <f aca="false">'4e ARR bridge'!B49</f>
+        <v>664</v>
+      </c>
+      <c r="E44" s="33" t="b">
+        <f aca="false">'4e ARR bridge'!B17</f>
         <v>1</v>
       </c>
     </row>
@@ -11520,16 +11594,16 @@
         <v>38</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>649</v>
+        <v>665</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="E45" s="31" t="b">
-        <f aca="false">'4e ARR bridge'!C49</f>
+        <v>666</v>
+      </c>
+      <c r="E45" s="33" t="b">
+        <f aca="false">'4e ARR bridge'!C17</f>
         <v>1</v>
       </c>
     </row>
@@ -11538,16 +11612,16 @@
         <v>39</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>651</v>
+        <v>667</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>652</v>
-      </c>
-      <c r="E46" s="31" t="b">
-        <f aca="false">'4e ARR bridge'!D49</f>
+        <v>668</v>
+      </c>
+      <c r="E46" s="33" t="b">
+        <f aca="false">'4e ARR bridge'!D17</f>
         <v>1</v>
       </c>
     </row>
@@ -11556,16 +11630,16 @@
         <v>40</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>653</v>
+        <v>669</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>654</v>
-      </c>
-      <c r="E47" s="31" t="b">
-        <f aca="false">'4f Margin'!C47</f>
+        <v>670</v>
+      </c>
+      <c r="E47" s="33" t="b">
+        <f aca="false">'4e ARR bridge'!B49</f>
         <v>1</v>
       </c>
     </row>
@@ -11574,16 +11648,16 @@
         <v>41</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>655</v>
+        <v>671</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>656</v>
-      </c>
-      <c r="E48" s="31" t="b">
-        <f aca="false">'4f Margin'!D47</f>
+        <v>672</v>
+      </c>
+      <c r="E48" s="33" t="b">
+        <f aca="false">'4e ARR bridge'!C49</f>
         <v>1</v>
       </c>
     </row>
@@ -11592,16 +11666,16 @@
         <v>42</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>657</v>
+        <v>673</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>658</v>
-      </c>
-      <c r="E49" s="31" t="b">
-        <f aca="false">'4f Margin'!E47</f>
+        <v>674</v>
+      </c>
+      <c r="E49" s="33" t="b">
+        <f aca="false">'4e ARR bridge'!D49</f>
         <v>1</v>
       </c>
     </row>
@@ -11610,16 +11684,16 @@
         <v>43</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>659</v>
+        <v>675</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>660</v>
-      </c>
-      <c r="E50" s="31" t="b">
-        <f aca="false">'4f Margin'!B56</f>
+        <v>676</v>
+      </c>
+      <c r="E50" s="33" t="b">
+        <f aca="false">'4f Margin'!C47</f>
         <v>1</v>
       </c>
     </row>
@@ -11628,16 +11702,16 @@
         <v>44</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>661</v>
+        <v>677</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>662</v>
-      </c>
-      <c r="E51" s="31" t="b">
-        <f aca="false">'4f Margin'!C56</f>
+        <v>678</v>
+      </c>
+      <c r="E51" s="33" t="b">
+        <f aca="false">'4f Margin'!D47</f>
         <v>1</v>
       </c>
     </row>
@@ -11646,16 +11720,16 @@
         <v>45</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>663</v>
+        <v>679</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>664</v>
-      </c>
-      <c r="E52" s="31" t="b">
-        <f aca="false">'4f Margin'!D56</f>
+        <v>680</v>
+      </c>
+      <c r="E52" s="33" t="b">
+        <f aca="false">'4f Margin'!E47</f>
         <v>1</v>
       </c>
     </row>
@@ -11664,16 +11738,16 @@
         <v>46</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>665</v>
+        <v>681</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="E53" s="31" t="b">
-        <f aca="false">'4f Margin'!E56</f>
+        <v>682</v>
+      </c>
+      <c r="E53" s="33" t="b">
+        <f aca="false">'4f Margin'!B56</f>
         <v>1</v>
       </c>
     </row>
@@ -11682,16 +11756,16 @@
         <v>47</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>667</v>
+        <v>683</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>668</v>
-      </c>
-      <c r="E54" s="31" t="b">
-        <f aca="false">'4f Margin'!E72</f>
+        <v>684</v>
+      </c>
+      <c r="E54" s="33" t="b">
+        <f aca="false">'4f Margin'!C56</f>
         <v>1</v>
       </c>
     </row>
@@ -11700,16 +11774,16 @@
         <v>48</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>669</v>
+        <v>685</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="E55" s="31" t="b">
-        <f aca="false">'4f Margin'!D80</f>
+        <v>686</v>
+      </c>
+      <c r="E55" s="33" t="b">
+        <f aca="false">'4f Margin'!D56</f>
         <v>1</v>
       </c>
     </row>
@@ -11718,16 +11792,16 @@
         <v>49</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>671</v>
+        <v>687</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>672</v>
-      </c>
-      <c r="E56" s="31" t="b">
-        <f aca="false">'4g Segments'!C31</f>
+        <v>688</v>
+      </c>
+      <c r="E56" s="33" t="b">
+        <f aca="false">'4f Margin'!E56</f>
         <v>1</v>
       </c>
     </row>
@@ -11736,16 +11810,16 @@
         <v>50</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>673</v>
+        <v>689</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>674</v>
-      </c>
-      <c r="E57" s="31" t="b">
-        <f aca="false">'4g Segments'!C32</f>
+        <v>690</v>
+      </c>
+      <c r="E57" s="33" t="b">
+        <f aca="false">'4f Margin'!E72</f>
         <v>1</v>
       </c>
     </row>
@@ -11754,16 +11828,16 @@
         <v>51</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>675</v>
+        <v>691</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>676</v>
-      </c>
-      <c r="E58" s="31" t="b">
-        <f aca="false">'4g Segments'!C33</f>
+        <v>692</v>
+      </c>
+      <c r="E58" s="33" t="b">
+        <f aca="false">'4f Margin'!D80</f>
         <v>1</v>
       </c>
     </row>
@@ -11772,16 +11846,16 @@
         <v>52</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>677</v>
+        <v>693</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="E59" s="31" t="b">
-        <f aca="false">'4g Segments'!C34</f>
+        <v>694</v>
+      </c>
+      <c r="E59" s="33" t="b">
+        <f aca="false">'4g Segments'!C31</f>
         <v>1</v>
       </c>
     </row>
@@ -11790,15 +11864,69 @@
         <v>53</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>679</v>
+        <v>695</v>
       </c>
       <c r="C60" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="E60" s="33" t="b">
+        <f aca="false">'4g Segments'!C32</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="E61" s="33" t="b">
+        <f aca="false">'4g Segments'!C33</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="E62" s="33" t="b">
+        <f aca="false">'4g Segments'!C34</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D60" s="2" t="s">
-        <v>680</v>
-      </c>
-      <c r="E60" s="31" t="b">
+      <c r="D63" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="E63" s="33" t="b">
         <f aca="false">Basis!F27</f>
         <v>1</v>
       </c>
@@ -21401,7 +21529,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:T35"/>
+  <dimension ref="A1:T66"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -22027,7 +22155,10 @@
         <v>357</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>12</v>
+        <v>358</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>359</v>
       </c>
       <c r="L29" s="22"/>
       <c r="M29" s="22"/>
@@ -22041,19 +22172,22 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>340</v>
+        <v>360</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>359</v>
+        <v>361</v>
+      </c>
+      <c r="C30" s="21" t="n">
+        <v>2025</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>361</v>
+        <v>339</v>
+      </c>
+      <c r="F30" s="28" t="n">
+        <v>0.98</v>
       </c>
       <c r="L30" s="22"/>
       <c r="M30" s="22"/>
@@ -22067,19 +22201,22 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="C31" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="E31" s="9" t="s">
         <v>339</v>
       </c>
-      <c r="B31" s="9" t="s">
-        <v>362</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>363</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>364</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>361</v>
+      <c r="F31" s="28" t="n">
+        <v>1.03</v>
       </c>
       <c r="L31" s="22"/>
       <c r="M31" s="22"/>
@@ -22092,6 +22229,24 @@
       <c r="T31" s="22"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="C32" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F32" s="28" t="n">
+        <v>1.02</v>
+      </c>
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
       <c r="N32" s="22"/>
@@ -22103,6 +22258,24 @@
       <c r="T32" s="22"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C33" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F33" s="28" t="n">
+        <v>0.98</v>
+      </c>
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
       <c r="N33" s="22"/>
@@ -22114,6 +22287,24 @@
       <c r="T33" s="22"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C34" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F34" s="28" t="n">
+        <v>0.97</v>
+      </c>
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
       <c r="N34" s="22"/>
@@ -22125,6 +22316,24 @@
       <c r="T34" s="22"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C35" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F35" s="28" t="n">
+        <v>0.94</v>
+      </c>
       <c r="L35" s="22"/>
       <c r="M35" s="22"/>
       <c r="N35" s="22"/>
@@ -22135,9 +22344,619 @@
       <c r="S35" s="22"/>
       <c r="T35" s="22"/>
     </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C36" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F36" s="28" t="n">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C37" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F37" s="28" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C38" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F38" s="28" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C39" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F39" s="28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C40" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F40" s="28" t="n">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C41" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F41" s="28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C42" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>374</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F42" s="28" t="n">
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C43" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="F43" s="28" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="C44" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F44" s="28" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="C45" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F45" s="28" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="B46" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="C46" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F46" s="28" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C47" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F47" s="28" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C48" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F48" s="28" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C49" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F49" s="28" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C50" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F50" s="28" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C51" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F51" s="28" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C52" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F52" s="28" t="n">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C53" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F53" s="28" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C54" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F54" s="28" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C55" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F55" s="28" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C56" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>374</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F56" s="28" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C57" s="21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="F57" s="28" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="I59" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="B60" s="23" t="n">
+        <f aca="false">MIN(F30:F43)</f>
+        <v>0.94</v>
+      </c>
+      <c r="C60" s="23" t="n">
+        <f aca="false">MAX(F30:F43)</f>
+        <v>1.07</v>
+      </c>
+      <c r="D60" s="23" t="n">
+        <f aca="false">MIN(F30:F32)</f>
+        <v>0.98</v>
+      </c>
+      <c r="E60" s="23" t="n">
+        <f aca="false">MAX(F30:F32)</f>
+        <v>1.03</v>
+      </c>
+      <c r="F60" s="23" t="n">
+        <f aca="false">G15</f>
+        <v>0.954434773207137</v>
+      </c>
+      <c r="G60" s="28" t="n">
+        <v>0.94</v>
+      </c>
+      <c r="H60" s="28" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="I60" s="15" t="b">
+        <f aca="false">AND(ABS(B60-G60)&lt;0.000001,ABS(C60-H60)&lt;0.000001)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="B61" s="23" t="n">
+        <f aca="false">MIN(F30:F43)</f>
+        <v>0.94</v>
+      </c>
+      <c r="C61" s="23" t="n">
+        <f aca="false">MAX(F30:F43)</f>
+        <v>1.07</v>
+      </c>
+      <c r="D61" s="23" t="n">
+        <f aca="false">MIN(F30:F32)</f>
+        <v>0.98</v>
+      </c>
+      <c r="E61" s="23" t="n">
+        <f aca="false">MAX(F30:F32)</f>
+        <v>1.03</v>
+      </c>
+      <c r="F61" s="23" t="n">
+        <f aca="false">G17</f>
+        <v>0.891995114698221</v>
+      </c>
+      <c r="G61" s="28" t="n">
+        <v>0.94</v>
+      </c>
+      <c r="H61" s="28" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="I61" s="15" t="b">
+        <f aca="false">AND(ABS(B61-G61)&lt;0.000001,ABS(C61-H61)&lt;0.000001)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B62" s="23" t="n">
+        <f aca="false">MIN(F44:F57)</f>
+        <v>0.83</v>
+      </c>
+      <c r="C62" s="23" t="n">
+        <f aca="false">MAX(F44:F57)</f>
+        <v>0.92</v>
+      </c>
+      <c r="D62" s="23" t="n">
+        <f aca="false">MIN(F44:F46)</f>
+        <v>0.9</v>
+      </c>
+      <c r="E62" s="23" t="n">
+        <f aca="false">MAX(F44:F46)</f>
+        <v>0.91</v>
+      </c>
+      <c r="F62" s="23" t="n">
+        <f aca="false">H15</f>
+        <v>0.887690505113145</v>
+      </c>
+      <c r="G62" s="28" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="H62" s="28" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="I62" s="15" t="b">
+        <f aca="false">AND(ABS(B62-G62)&lt;0.000001,ABS(C62-H62)&lt;0.000001)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="29" t="s">
+        <v>384</v>
+      </c>
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
+      <c r="D64" s="29"/>
+      <c r="E64" s="29"/>
+      <c r="F64" s="29"/>
+      <c r="G64" s="29"/>
+      <c r="H64" s="29"/>
+      <c r="I64" s="29"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="29"/>
+      <c r="B65" s="29"/>
+      <c r="C65" s="29"/>
+      <c r="D65" s="29"/>
+      <c r="E65" s="29"/>
+      <c r="F65" s="29"/>
+      <c r="G65" s="29"/>
+      <c r="H65" s="29"/>
+      <c r="I65" s="29"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="29"/>
+      <c r="B66" s="29"/>
+      <c r="C66" s="29"/>
+      <c r="D66" s="29"/>
+      <c r="E66" s="29"/>
+      <c r="F66" s="29"/>
+      <c r="G66" s="29"/>
+      <c r="H66" s="29"/>
+      <c r="I66" s="29"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="L24:T35"/>
+    <mergeCell ref="A64:I66"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22165,22 +22984,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>365</v>
+        <v>385</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>366</v>
+        <v>386</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>367</v>
+        <v>387</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>368</v>
+        <v>388</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22199,7 +23018,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>369</v>
+        <v>389</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>29005683.6</v>
@@ -22215,7 +23034,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>370</v>
+        <v>390</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>5003640.48</v>
@@ -22229,7 +23048,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>371</v>
+        <v>391</v>
       </c>
       <c r="B9" s="11" t="n">
         <v>360985.44</v>
@@ -22243,7 +23062,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>372</v>
+        <v>392</v>
       </c>
       <c r="B10" s="11" t="n">
         <v>0</v>
@@ -22257,7 +23076,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>373</v>
+        <v>393</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>0</v>
@@ -22271,7 +23090,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>374</v>
+        <v>394</v>
       </c>
       <c r="B12" s="11" t="n">
         <v>-79064.4</v>
@@ -22285,7 +23104,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>375</v>
+        <v>395</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>0</v>
@@ -22299,7 +23118,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>376</v>
+        <v>396</v>
       </c>
       <c r="B14" s="11" t="n">
         <v>-1509902.52</v>
@@ -22313,7 +23132,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>377</v>
+        <v>397</v>
       </c>
       <c r="B15" s="14" t="n">
         <f aca="false">SUM(B7:B14)</f>
@@ -22330,7 +23149,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>378</v>
+        <v>398</v>
       </c>
       <c r="B16" s="12" t="n">
         <f aca="false">SUMIFS('4a Revenue quality'!$B$15:$B$18,'4a Revenue quality'!$A$15:$A$18,2023)</f>
@@ -22364,21 +23183,21 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>379</v>
+        <v>399</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>380</v>
+        <v>400</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>381</v>
+        <v>401</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>382</v>
+        <v>402</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>383</v>
+        <v>403</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>61</v>
@@ -22386,7 +23205,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>369</v>
+        <v>389</v>
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">0</f>
@@ -22407,7 +23226,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>370</v>
+        <v>390</v>
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">MIN(SUM($D$7:D7),SUM($D$7:D7)+D8)</f>
@@ -22428,7 +23247,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>371</v>
+        <v>391</v>
       </c>
       <c r="B23" s="12" t="n">
         <f aca="false">MIN(SUM($D$7:D8),SUM($D$7:D8)+D9)</f>
@@ -22449,7 +23268,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>372</v>
+        <v>392</v>
       </c>
       <c r="B24" s="12" t="n">
         <f aca="false">MIN(SUM($D$7:D9),SUM($D$7:D9)+D10)</f>
@@ -22470,7 +23289,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>373</v>
+        <v>393</v>
       </c>
       <c r="B25" s="12" t="n">
         <f aca="false">MIN(SUM($D$7:D10),SUM($D$7:D10)+D11)</f>
@@ -22491,7 +23310,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>374</v>
+        <v>394</v>
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">MIN(SUM($D$7:D11),SUM($D$7:D11)+D12)</f>
@@ -22510,7 +23329,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="22" t="s">
-        <v>384</v>
+        <v>404</v>
       </c>
       <c r="K26" s="22"/>
       <c r="L26" s="22"/>
@@ -22524,7 +23343,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>375</v>
+        <v>395</v>
       </c>
       <c r="B27" s="12" t="n">
         <f aca="false">MIN(SUM($D$7:D12),SUM($D$7:D12)+D13)</f>
@@ -22555,7 +23374,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>376</v>
+        <v>396</v>
       </c>
       <c r="B28" s="12" t="n">
         <f aca="false">MIN(SUM($D$7:D13),SUM($D$7:D13)+D14)</f>
@@ -22586,7 +23405,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>377</v>
+        <v>397</v>
       </c>
       <c r="B29" s="12" t="n">
         <f aca="false">0</f>
@@ -22641,7 +23460,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
-        <v>385</v>
+        <v>405</v>
       </c>
       <c r="J32" s="22"/>
       <c r="K32" s="22"/>
@@ -22680,7 +23499,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>386</v>
+        <v>406</v>
       </c>
       <c r="B34" s="11" t="n">
         <v>28232151.64</v>
@@ -22704,7 +23523,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>370</v>
+        <v>390</v>
       </c>
       <c r="B35" s="11" t="n">
         <v>2884583.65</v>
@@ -22728,7 +23547,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>387</v>
+        <v>407</v>
       </c>
       <c r="B36" s="11" t="n">
         <v>2039767.82</v>
@@ -22752,7 +23571,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>371</v>
+        <v>391</v>
       </c>
       <c r="B37" s="11" t="n">
         <v>196902.61</v>
@@ -22776,7 +23595,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>372</v>
+        <v>392</v>
       </c>
       <c r="B38" s="11" t="n">
         <v>0</v>
@@ -22800,7 +23619,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>373</v>
+        <v>393</v>
       </c>
       <c r="B39" s="11" t="n">
         <v>0</v>
@@ -22824,7 +23643,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>388</v>
+        <v>408</v>
       </c>
       <c r="B40" s="11" t="n">
         <v>-3911.95</v>
@@ -22838,7 +23657,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>374</v>
+        <v>394</v>
       </c>
       <c r="B41" s="11" t="n">
         <v>-76395.5</v>
@@ -22852,7 +23671,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>375</v>
+        <v>395</v>
       </c>
       <c r="B42" s="11" t="n">
         <v>0</v>
@@ -22866,7 +23685,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>376</v>
+        <v>396</v>
       </c>
       <c r="B43" s="11" t="n">
         <v>-1326723.42</v>
@@ -22880,7 +23699,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>389</v>
+        <v>409</v>
       </c>
       <c r="B44" s="11" t="n">
         <v>52150.89</v>
@@ -22894,7 +23713,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>390</v>
+        <v>410</v>
       </c>
       <c r="B45" s="11" t="n">
         <v>194344.21</v>
@@ -22908,7 +23727,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>391</v>
+        <v>411</v>
       </c>
       <c r="B46" s="11" t="n">
         <v>0</v>
@@ -22939,7 +23758,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>392</v>
+        <v>412</v>
       </c>
       <c r="B48" s="12" t="n">
         <f aca="false">SUMIFS('4a Revenue quality'!$F$7:$F$10,'4a Revenue quality'!$A$7:$A$10,2023)</f>
@@ -22973,7 +23792,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>393</v>
+        <v>413</v>
       </c>
       <c r="B50" s="12" t="n">
         <f aca="false">SUM(B35:B44)</f>
@@ -22990,7 +23809,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>394</v>
+        <v>414</v>
       </c>
       <c r="B51" s="12" t="n">
         <f aca="false">SUM(B45:B46)</f>

</xml_diff>